<commit_message>
Update references and project documentation
</commit_message>
<xml_diff>
--- a/Anatomy_Extraction_Master_Tracker_v2.xlsx
+++ b/Anatomy_Extraction_Master_Tracker_v2.xlsx
@@ -1052,7 +1052,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U6"/>
+  <dimension ref="A1:U7"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="5"/>
   <sheetData>
     <row r="1">
@@ -1193,9 +1193,14 @@
           <t>5,8,17</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>ch7: 235-267; ch2: 51-65, 82; ch6: 216-221; ch17: 624-628</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>corneal_epithelium.json</t>
+          <t>corneal-epithelium.json</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -1205,7 +1210,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done (manual, Wolff ch.2/6/7/17 + StatPearls)</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -1215,7 +1220,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (validate.py, 2026-10-17)</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -1250,7 +1255,12 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Filename fixed to match repo (corneal-epithelium.json); supporting material from ch2 (limbus/conjunctiva), ch6 (dimensions, stem cells) and ch17 (development) in addition to ch7; pages 233-234 and 259-265 of ch7 not yet provided - definition supported by ch6 p.216; revalidated 2026-10-17 after bilingual keyword surface + alias (v1.0.1)</t>
         </is>
       </c>
     </row>
@@ -1267,7 +1277,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Bowman's Layer</t>
+          <t>"Bowman's Layer"</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1285,9 +1295,14 @@
           <t>5,8,17</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>ch7: 247-249; ch17: 627-628</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>bowmans_layer.json</t>
+          <t>bowmans-layer.json</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -1297,7 +1312,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done (manual, Wolff ch.7/17 + StatPearls)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -1307,7 +1322,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (validate.py, 2026-10-17)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -1342,7 +1357,12 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Extracted from already-read pages: ch7 247-249 (structure) + ch17 627-628 (development, synthesised by basal epithelial cells). 8/8 fields documented with page sources; statpearls only for avascular statements. Awaiting user PR.</t>
         </is>
       </c>
     </row>
@@ -1377,9 +1397,14 @@
           <t>5,8,17</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>ch7: 249-252, 266, 268-270; ch6: 216-218</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>stroma.json</t>
+          <t>corneal-stroma.json</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -1389,7 +1414,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done (manual, Wolff ch.7/6 + StatPearls)</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -1399,7 +1424,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (validate.py, 2026-10-17)</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -1434,7 +1459,12 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Extracted from already-read pages: ch7 249-252 (structure), 266 (transparency), 268-270 (limbal transition, ground substance) + ch6 216-218 (dimensions). Richest card (~970 tokens). 8/8 fields documented. Awaiting user PR.</t>
         </is>
       </c>
     </row>
@@ -1451,7 +1481,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Descemet's Membrane</t>
+          <t>"Descemet's Membrane"</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1469,9 +1499,14 @@
           <t>5,8,17</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>ch7: 251-258; ch17: 626; ch8: 284, 286</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>descemets_membrane.json</t>
+          <t>descemets-membrane.json</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1481,7 +1516,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done (manual, Wolff ch.7/17/8 + StatPearls)</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -1491,7 +1526,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (validate.py, 2026-10-17)</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -1526,7 +1561,12 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Extracted from already-read pages: ch7 251-255 (membrane), 256-257 (endothelial attachment) + ch17 626 (development) + ch8 284/286 (Schwalbe/angle). 8/8 fields documented; innervation = not_available (posterior stromal nerves end before reaching it, ch7 p.267). Awaiting user PR.</t>
         </is>
       </c>
     </row>
@@ -1588,7 +1628,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Yes (validate.py, 2026-10-16)</t>
+          <t>Yes (validate.py, 2026-10-17)</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1628,7 +1668,109 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>Filename fixed to match repo (corneal-endothelium.json). Reference registry corrected: authors are Bron, Tripathi &amp; Tripathi, Chapman &amp; Hall Medical, 8th ed., 1997 (verified vs title/copyright pages). innervation field = not_available, re-check ch.7.1 during full-text extraction.</t>
+          <t>Filename fixed to match repo (corneal-endothelium.json). Reference registry corrected: authors are Bron, Tripathi &amp; Tripathi, Chapman &amp; Hall Medical, 8th ed., 1997 (verified vs title/copyright pages). innervation field = not_available, re-check ch.7.1 during full-text extraction.; keywords v1.1.1 (Arabic + cell density/deturgescence), revalidated 2026-10-17; pages 259-265 still outstanding - nerves pages 266-267 (read) support the posterior-stroma-only innervation pattern</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CONJ-001</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Conjunctiva</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Bulbar Conjunctiva</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2, 6</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>ch2: 51-65, 66-71, 82; ch6: 222</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>bulbar-conjunctiva.json</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff ch.2+ch.6 + StatPearls)</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 2026-10-17)</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>First non-cornea entity, built in parallel with the retina assignment. Extracted from ch2 51-65 re-read in full + p82 (tear film); StatPearls NBK519502 read in full - adds named sensory innervation (supraorbital/supratrochlear/infratrochlear/infraorbital/lacrimal/long ciliary), Tenon's binding and ~33 um thickness, arcades + posterior conjunctival arteries + watershed 3-4 mm from limbus, conjunctivochalasis, staining/grading (Oxford/NEI). venous_drainage = not_available (no named bulbar conjunctival veins in either source). | v1.1.0 enrichment: Wolff ch2 pp66-71 read in full + ch6 p222 - venous_drainage filled from THE CONJUNCTIVAL VEINS p69 (palpebral veins drain posterior bulbar conjunctiva to levator/superior rectus veins then ophthalmic; anterior conjunctival veins via perilimbal venous circle -&gt; radial episcleral collecting veins -&gt; rectus muscle veins); arterial supply upgraded to 4 named sources p67 + episcleral hairpin bend p68 + deep ciliary circle and limbal capillary network p69; redness differential conjunctivitis vs ciliary injection p68-69; lymphatics lateral-&gt;parotid / medial-&gt;submandibular p69-70; end bulbs of Krause p70; lymphoid layer 50-70 um + Krause 42/6-8 + Wolfring 2-5/2 p66-67; plica recess 2 mm + limbus widths 2/1.5 mm p71/p222. Awaiting user PR. | v1.2.0 StatPearls deep-mining (NBK519502 full text re-mined): embryology - ocular surface ectoderm origin shared with corneal and limbal epithelia; no muscle attaches directly, rectus insertions lie deep to bulbar conjunctiva; goblet cells greatest near fornices (inferior+medial, medial canthus) decreasing away; forniceal lymphoid patches mostly suppressor T-cells; anterior ciliary arteries traced to ophthalmic artery + marginal arcades supply palpebral conjunctiva and fornices; lissamine green better tolerated than rose bengal. Related StatPearls articles identified (Pterygium NBK558907 / Pinguecula NBK558965 / Subconjunctival Hemorrhage NBK551666) but NOT read this session (NCBI reCAPTCHA + Europe PMC outage) - not cited per unread-source rule. Awaiting user PR. | v1.3.0 enrichment: three related StatPearls articles read in full (Pterygium NBK558907, Pinguecula NBK558965, Subconjunctival Hemorrhage NBK551666) - 28 facts added: blood_supply +4 (nasal 2-vs-1 anterior ciliary asymmetry -&gt; greater nasal hyperaemia; dense capillary network perfusing epithelium and stroma; fine unsupported fragile capillaries; vessel distribution in conjunctival vs ciliary congestion); location +3 (interpalpebral UV belt and pterygium belt 30-37 deg; 3 &amp; 9 o'clock perilimbal clustering with nasal predilection; larger temporal surface -&gt; inferotemporal haemorrhage pooling); histology_summary +8 (elastotic degeneration - elastin-staining, elastase-resistant, with fat/calcified globules; AGE deposits; lymphoplasmacytic infiltrate; racial melanosis; contact-lens friction degeneration; conjunctivo-Tenon potential space; transient goblet-cell loss and BM irregularity; limited lymphatic drainage); clinical_importance +13 (pterygium origin + limbal barrier/conjunctivalization + peripheral light focusing; superotemporal autograft donor site + BSS hydrodissection + 0.5 mm limbal graft + 6-month regeneration; tear-film instability + inflammatory mediators; systemic window - Gaucher cells, OSSN/melanoma feeder vessels; SCH natural history 7-14 days with colour sequence; Valsalva/rubbing precipitants; hypertension/anticoagulants/10% recurrence/fornix haemorrhage -&gt; basilar skull fracture; infant NAT red flags + 1-2% newborns; vascular mimics); 3 reference entries appended (registry now 9 sources); card 2,572 -&gt; 3580 words. Awaiting user PR.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update knowledge base and anatomy data
</commit_message>
<xml_diff>
--- a/Anatomy_Extraction_Master_Tracker_v2.xlsx
+++ b/Anatomy_Extraction_Master_Tracker_v2.xlsx
@@ -1052,7 +1052,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U7"/>
+  <dimension ref="A1:U9"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="5"/>
   <sheetData>
     <row r="1">
@@ -1771,6 +1771,210 @@
       <c r="U7" t="inlineStr">
         <is>
           <t>First non-cornea entity, built in parallel with the retina assignment. Extracted from ch2 51-65 re-read in full + p82 (tear film); StatPearls NBK519502 read in full - adds named sensory innervation (supraorbital/supratrochlear/infratrochlear/infraorbital/lacrimal/long ciliary), Tenon's binding and ~33 um thickness, arcades + posterior conjunctival arteries + watershed 3-4 mm from limbus, conjunctivochalasis, staining/grading (Oxford/NEI). venous_drainage = not_available (no named bulbar conjunctival veins in either source). | v1.1.0 enrichment: Wolff ch2 pp66-71 read in full + ch6 p222 - venous_drainage filled from THE CONJUNCTIVAL VEINS p69 (palpebral veins drain posterior bulbar conjunctiva to levator/superior rectus veins then ophthalmic; anterior conjunctival veins via perilimbal venous circle -&gt; radial episcleral collecting veins -&gt; rectus muscle veins); arterial supply upgraded to 4 named sources p67 + episcleral hairpin bend p68 + deep ciliary circle and limbal capillary network p69; redness differential conjunctivitis vs ciliary injection p68-69; lymphatics lateral-&gt;parotid / medial-&gt;submandibular p69-70; end bulbs of Krause p70; lymphoid layer 50-70 um + Krause 42/6-8 + Wolfring 2-5/2 p66-67; plica recess 2 mm + limbus widths 2/1.5 mm p71/p222. Awaiting user PR. | v1.2.0 StatPearls deep-mining (NBK519502 full text re-mined): embryology - ocular surface ectoderm origin shared with corneal and limbal epithelia; no muscle attaches directly, rectus insertions lie deep to bulbar conjunctiva; goblet cells greatest near fornices (inferior+medial, medial canthus) decreasing away; forniceal lymphoid patches mostly suppressor T-cells; anterior ciliary arteries traced to ophthalmic artery + marginal arcades supply palpebral conjunctiva and fornices; lissamine green better tolerated than rose bengal. Related StatPearls articles identified (Pterygium NBK558907 / Pinguecula NBK558965 / Subconjunctival Hemorrhage NBK551666) but NOT read this session (NCBI reCAPTCHA + Europe PMC outage) - not cited per unread-source rule. Awaiting user PR. | v1.3.0 enrichment: three related StatPearls articles read in full (Pterygium NBK558907, Pinguecula NBK558965, Subconjunctival Hemorrhage NBK551666) - 28 facts added: blood_supply +4 (nasal 2-vs-1 anterior ciliary asymmetry -&gt; greater nasal hyperaemia; dense capillary network perfusing epithelium and stroma; fine unsupported fragile capillaries; vessel distribution in conjunctival vs ciliary congestion); location +3 (interpalpebral UV belt and pterygium belt 30-37 deg; 3 &amp; 9 o'clock perilimbal clustering with nasal predilection; larger temporal surface -&gt; inferotemporal haemorrhage pooling); histology_summary +8 (elastotic degeneration - elastin-staining, elastase-resistant, with fat/calcified globules; AGE deposits; lymphoplasmacytic infiltrate; racial melanosis; contact-lens friction degeneration; conjunctivo-Tenon potential space; transient goblet-cell loss and BM irregularity; limited lymphatic drainage); clinical_importance +13 (pterygium origin + limbal barrier/conjunctivalization + peripheral light focusing; superotemporal autograft donor site + BSS hydrodissection + 0.5 mm limbal graft + 6-month regeneration; tear-film instability + inflammatory mediators; systemic window - Gaucher cells, OSSN/melanoma feeder vessels; SCH natural history 7-14 days with colour sequence; Valsalva/rubbing precipitants; hypertension/anticoagulants/10% recurrence/fornix haemorrhage -&gt; basilar skull fracture; infant NAT red flags + 1-2% newborns; vascular mimics); 3 reference entries appended (registry now 9 sources); card 2,572 -&gt; 3580 words. Awaiting user PR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CONJ-002</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Conjunctiva</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Palpebral Conjunctiva</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2, 4</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>ch2: 39, 51-53, 66-67, 69-70; ch4: 146, 148, 150</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>palpebral-conjunctiva.json</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff ch2 + ch4 + StatPearls x3)</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 2026-10-19)</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>v1.0.0 first extraction. Sources read directly (visual): printed 39 (palpebral conjunctiva firmly adherent to tarsus; septum orbitale piercings; inferior Mueller palpebral muscle visible through conjunctiva), 51 (THE PALPEBRAL CONJUNCTIVA: marginal/tarsal/orbital zones in full; conjunctival sac 7-30 uL), 52 (Fig 2.30 sac zones + dimensions), 53 (mucocutaneous junction; goblet cells beyond subtarsal fold, Kessing 1968), 66 (Wolfring glands at tarsal borders; lymphoid layer 50-70 um absent from marginal zone), 67 (4 arterial sources; peripheral + marginal tarsal arcades; papillae only at limbus and marginal conjunctiva), 69 (palpebral veins drain tarsal conjunctiva via levator plexus to ophthalmic; redness patterns), 70 (nerve sources = lid nerves; end bulbs of Krause 20-100 um), 144-149 (Muller superior palpebral muscle in full: 3 mm elevation, sympathetic, Horner 3-4 mm, phenylephrine/guanethidine access; Fig 4.38 label 10; inferior rectus expansion deep to inferior fornix and palpebral conjunctiva, lid lowered 2 mm; suspensory ligaments of fornices start). Printed 51-53, 66-67, 69-70 read from page images recovered from the previous session history; printed 39 and 144-149 from owner-supplied PDFs. validate 7/7, pytest 10+14. Awaiting user PR. | v1.1.0 (2026-10-19): enrichment from 4 fully-read sources - Wolff printed 150 (PDF 160, visual read), statpearls_conjunctiva NBK519502 (re-read for palpebral/fornix sections), statpearls_muller_muscle NBK540964 NEW (2024-10-05), statpearls_conjunctivitis NBK541034 NEW (2026-09-08). Added: lid layering (skin-&gt;orbicularis-&gt;tarsus-&gt;palpebral conjunctiva); Muller geometry 15-20x10mm (Wolff) vs ~15x10mm (StatPearls) + pretrasal-space limitation + lacrimal-gland palpebral-lobe slip + capsulopalpebral muscle (of Hesser) parts; epithelium 3-5 strata concordance + substantia propria uniqueness; regional sensory map (supraorbital/supratrochlear/infratrochlear superior, infraorbital inferior, lacrimal lateral, long ciliary circumcorneal) + sympathetic route via internal carotid plexus/ophthalmic artery; papillary (fibrovascular core, central vessels) vs follicular (germinal centres, no central vessels, inferior predominance); tarsal disease geography GPC/FES/VKC/AKC/trachoma (Arlt line, Herbert pits); +2mm sympathetic elevation, TED retraction, Horner paralysis concordance; MMCR technique + meta-analysis (no MRD difference, overcorrection/reoperations higher with levator advancement). 1,428-&gt;2,417 words. 48/48 source-quote checks passed. validate 8/8 + pytest 10+14. references.json 9-&gt;12.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>CONJ-003</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Conjunctiva</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Conjunctival Fornix</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2, 4</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>ch2: 51-53, 66-67, 69-70, 82; ch4: 145, 148, 150</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>conjunctival-fornix.json</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff ch2 + ch4 + StatPearls x3)</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 2026-10-19)</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>v1.0.0 first extraction. Sources read directly (visual): printed 51 (2.6 THE CONJUNCTIVA: sac 7 microlitre / 30 microlitre; three regions palpebral-bulbar-fornical), 52 (THE CONJUNCTIVAL FORNIX complete: annular cul-de-sac; superior 8-10mm from limbus reaching orbital margin, inferior 8mm, lateral 5mm from surface / 14mm from limbus just posterior to equator, medial shallowest; Fig 2.30 Whitnall 1921 lid-margin 13/9/5 and from-limbus 8-10/14/7; areolar adherence continuous with levator/rectus sheath expansions deepening fornices; glands of Krause + palpebral muscles of Mueller; orbital fat in intertendinous intervals behind fornices -&gt; basal cranial fracture haemorrhage to limbus; whole fornix well vascularized with venous plexus + IR/IO aponeurotic expansions visible inferiorly; incision planes), 67 (peripheral tarsal arcade runs in tarsal plate, fornix and proximal bulbar conjunctiva; ascending branches over fornix -&gt; posterior conjunctival arteries anastomosing ~4mm from limbus; lower-lid peripheral arcade often absent -&gt; marginal arcade or muscular arteries to inferior rectus), 70 (conjunctival innervation same sources as lids; lacrimal/infratrochlear supply larger conjunctival proportion; end bulbs of Krause distinct from fornix glands of Krause), 82 (DISTRIBUTION OF THE TEARS: fornices 4.5 microlitre vs preocular film 1.1 microlitre vs marginal strips), ch4 145 (sheath of levator attached to superior rectus sheath; intervening tissue gains attachment to upper conjunctival fornix, Fig 2.49) + 148 (inferior rectus expansion deep to inferior fornix separated by unstriated inferior palpebral muscle; lid lowered 2mm lashes everted; SUSPENSORY LIGAMENTS OF THE FORNICES opens: fibrous tissue between SR and levator continues forward to upper fornix). Owner's text census of 'conjunctival fornix' (PDF 61/62/92/155) fully honoured - all four hits re-read first-hand. Printed 150 (continuation of SUSPENSORY LIGAMENTS OF THE FORNICES) not yet read - flagged for v1.1.0, not cited. | v1.1.0 (2026-10-19): THE missing page arrived and was read visually - printed 150 (PDF 160): superior suspensory ligament of the fornix (tissue between levator and SR sheaths; cut during ptosis surgery -&gt; conjunctival prolapse, Collin 1983) + inferior suspensory ligament (extension of lid-retractor fibrous tissue; involutional laxity -&gt; lower fornix shallowed, Figs 4.37/4.43) + Muller passes just behind the fornix (surgical landmark). From StatPearls: goblet-cell density maximal closest to the fornix + lymphocyte patches mostly suppressor T-cells forming CALT (NBK519502); normal fornix depths 15.3mm superior / 10.9mm inferior (Khan 2014, NBK582141 NEW) with measurement-convention caveat vs Whitnall; GFS full clinical block - deep-fornix reservoir from aponeurosis degradation, S aureus/P aeruginosa/S marcescens, exudate feedback loop, 10% povidone-iodine forniceal swabs (curative 97yo), resection 4-10mm, MMCR maximal 10-12mm &gt; limited 6-8mm, no tear-production deficits, CT free-air sign (NBK582141); double lid eversion for GFS protein clumps + fornix reconstruction mandatory if non-resolving + inferior-fornix follicles (inclusion conjunctivitis) + cicatricial shortening in MMP/AKC (NBK541034 NEW). 1,062-&gt;1,766 words. 48/48 source-quote checks. validate 8/8 + pytest 10+14. references.json 9-&gt;12.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Enrich all 10 retina cards with Wolff Ch.17 development facts (v1.1.0) + tracker RET rows
- Ch.17 'Development of the Human Eye' (printed pp.646-655, file 16.pdf):
  page-referenced developmental passages appended to histology_summary
  of every retina card; ch17 sources added to reference blocks
- Tracker: RET-001..010 rows added (19 rows total), ch17 recorded as
  supporting chapter
- validate 18/18, pytest 10 passed + 14 subtests
</commit_message>
<xml_diff>
--- a/Anatomy_Extraction_Master_Tracker_v2.xlsx
+++ b/Anatomy_Extraction_Master_Tracker_v2.xlsx
@@ -1052,7 +1052,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U9"/>
+  <dimension ref="A1:U19"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="5"/>
   <sheetData>
     <row r="1">
@@ -1975,6 +1975,1076 @@
       <c r="U9" t="inlineStr">
         <is>
           <t>v1.0.0 first extraction. Sources read directly (visual): printed 51 (2.6 THE CONJUNCTIVA: sac 7 microlitre / 30 microlitre; three regions palpebral-bulbar-fornical), 52 (THE CONJUNCTIVAL FORNIX complete: annular cul-de-sac; superior 8-10mm from limbus reaching orbital margin, inferior 8mm, lateral 5mm from surface / 14mm from limbus just posterior to equator, medial shallowest; Fig 2.30 Whitnall 1921 lid-margin 13/9/5 and from-limbus 8-10/14/7; areolar adherence continuous with levator/rectus sheath expansions deepening fornices; glands of Krause + palpebral muscles of Mueller; orbital fat in intertendinous intervals behind fornices -&gt; basal cranial fracture haemorrhage to limbus; whole fornix well vascularized with venous plexus + IR/IO aponeurotic expansions visible inferiorly; incision planes), 67 (peripheral tarsal arcade runs in tarsal plate, fornix and proximal bulbar conjunctiva; ascending branches over fornix -&gt; posterior conjunctival arteries anastomosing ~4mm from limbus; lower-lid peripheral arcade often absent -&gt; marginal arcade or muscular arteries to inferior rectus), 70 (conjunctival innervation same sources as lids; lacrimal/infratrochlear supply larger conjunctival proportion; end bulbs of Krause distinct from fornix glands of Krause), 82 (DISTRIBUTION OF THE TEARS: fornices 4.5 microlitre vs preocular film 1.1 microlitre vs marginal strips), ch4 145 (sheath of levator attached to superior rectus sheath; intervening tissue gains attachment to upper conjunctival fornix, Fig 2.49) + 148 (inferior rectus expansion deep to inferior fornix separated by unstriated inferior palpebral muscle; lid lowered 2mm lashes everted; SUSPENSORY LIGAMENTS OF THE FORNICES opens: fibrous tissue between SR and levator continues forward to upper fornix). Owner's text census of 'conjunctival fornix' (PDF 61/62/92/155) fully honoured - all four hits re-read first-hand. Printed 150 (continuation of SUSPENSORY LIGAMENTS OF THE FORNICES) not yet read - flagged for v1.1.0, not cited. | v1.1.0 (2026-10-19): THE missing page arrived and was read visually - printed 150 (PDF 160): superior suspensory ligament of the fornix (tissue between levator and SR sheaths; cut during ptosis surgery -&gt; conjunctival prolapse, Collin 1983) + inferior suspensory ligament (extension of lid-retractor fibrous tissue; involutional laxity -&gt; lower fornix shallowed, Figs 4.37/4.43) + Muller passes just behind the fornix (surgical landmark). From StatPearls: goblet-cell density maximal closest to the fornix + lymphocyte patches mostly suppressor T-cells forming CALT (NBK519502); normal fornix depths 15.3mm superior / 10.9mm inferior (Khan 2014, NBK582141 NEW) with measurement-convention caveat vs Whitnall; GFS full clinical block - deep-fornix reservoir from aponeurosis degradation, S aureus/P aeruginosa/S marcescens, exudate feedback loop, 10% povidone-iodine forniceal swabs (curative 97yo), resection 4-10mm, MMCR maximal 10-12mm &gt; limited 6-8mm, no tear-production deficits, CT free-air sign (NBK582141); double lid eversion for GFS protein clumps + fornix reconstruction mandatory if non-resolving + inferior-fornix follicles (inclusion conjunctivitis) + cicatricial shortening in MMP/AKC (NBK541034 NEW). 1,062-&gt;1,766 words. 48/48 source-quote checks. validate 8/8 + pytest 10+14. references.json 9-&gt;12.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>RET-001</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Retina</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Retinal Pigment Epithelium</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>ch14: 454, 460, 461, 462, 463, 464; ch17: 654, 655 (ch17 = development section, pp.646-655)</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>retinal-pigment-epithelium.json</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff ch.14 + ch.17 development)</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>v1.1.0; enriched 2026-10-23 with developmental facts from Wolff ch.17 (Development of the Human Eye, pp.646-655, uploaded file 16.pdf) - each fact page-referenced; validate 18/18, pytest 10+14 green</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>RET-002</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Retina</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>External Limiting Membrane</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>ch14: 463, 470, 471, 472, 473; ch17: 647, 649, 651 (ch17 = development section, pp.646-655)</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>external-limiting-membrane.json</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff ch.14 + ch.17 development)</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>v1.1.0; enriched 2026-10-23 with developmental facts from Wolff ch.17 (Development of the Human Eye, pp.646-655, uploaded file 16.pdf) - each fact page-referenced; validate 18/18, pytest 10+14 green</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>RET-003</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Retina</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Photoreceptor Layer (Rods and Cones)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>ch14: 460, 461, 463, 464, 465, 466, 467, 468, 469, 470, 471, 472, 473; ch17: 649, 650, 651, 652 (ch17 = development section, pp.646-655)</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>photoreceptor-layer.json</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff ch.14 + ch.17 development)</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>v1.1.0; enriched 2026-10-23 with developmental facts from Wolff ch.17 (Development of the Human Eye, pp.646-655, uploaded file 16.pdf) - each fact page-referenced; validate 18/18, pytest 10+14 green</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>RET-004</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Retina</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Outer Nuclear Layer</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>ch14: 463, 464, 467, 471, 473, 474; ch17: 650, 651, 652 (ch17 = development section, pp.646-655)</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>outer-nuclear-layer.json</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff ch.14 + ch.17 development)</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>v1.1.0; enriched 2026-10-23 with developmental facts from Wolff ch.17 (Development of the Human Eye, pp.646-655, uploaded file 16.pdf) - each fact page-referenced; validate 18/18, pytest 10+14 green</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>RET-005</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Retina</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Outer Plexiform Layer</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>ch14: 463, 474, 475, 476, 477; ch17: 650, 651, 652 (ch17 = development section, pp.646-655)</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>outer-plexiform-layer.json</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff ch.14 + ch.17 development)</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>v1.1.0; enriched 2026-10-23 with developmental facts from Wolff ch.17 (Development of the Human Eye, pp.646-655, uploaded file 16.pdf) - each fact page-referenced; validate 18/18, pytest 10+14 green</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>RET-006</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Retina</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Inner Nuclear Layer</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>ch3: 99, 101; ch14: 476, 477, 478, 479, 480, 481, 482, 483, 484; ch15: 491, 492; ch17: 650, 651, 652 (ch17 = development section, pp.646-655)</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>inner-nuclear-layer.json</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff ch.14 + ch.17 development)</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>v1.1.0; enriched 2026-10-23 with developmental facts from Wolff ch.17 (Development of the Human Eye, pp.646-655, uploaded file 16.pdf) - each fact page-referenced; validate 18/18, pytest 10+14 green</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>RET-007</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Retina</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Inner Plexiform Layer</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>ch3: 99, 101; ch14: 480, 482, 483, 484; ch15: 491, 492; ch17: 647, 648, 652 (ch17 = development section, pp.646-655)</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>inner-plexiform-layer.json</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff ch.14 + ch.17 development)</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>v1.1.0; enriched 2026-10-23 with developmental facts from Wolff ch.17 (Development of the Human Eye, pp.646-655, uploaded file 16.pdf) - each fact page-referenced; validate 18/18, pytest 10+14 green</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>RET-008</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Retina</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Ganglion Cell Layer</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>ch3: 99, 101; ch14: 484, 485, 486; ch15: 491, 492; ch17: 646, 647, 648, 649, 652 (ch17 = development section, pp.646-655)</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>ganglion-cell-layer.json</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff ch.14 + ch.17 development)</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>v1.1.0; enriched 2026-10-23 with developmental facts from Wolff ch.17 (Development of the Human Eye, pp.646-655, uploaded file 16.pdf) - each fact page-referenced; validate 18/18, pytest 10+14 green</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>RET-009</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Retina</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Nerve Fibre Layer</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>ch3: 99, 101; ch14: 485, 486, 487; ch15: 491, 492; ch17: 648, 651, 652 (ch17 = development section, pp.646-655)</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>nerve-fibre-layer.json</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff ch.14 + ch.17 development)</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>v1.1.0; enriched 2026-10-23 with developmental facts from Wolff ch.17 (Development of the Human Eye, pp.646-655, uploaded file 16.pdf) - each fact page-referenced; validate 18/18, pytest 10+14 green</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>RET-010</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Retina</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Internal Limiting Membrane</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>ch14: 463, 485, 487, 488; ch15: 490; ch17: 647 (ch17 = development section, pp.646-655)</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>internal-limiting-membrane.json</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff ch.14 + ch.17 development)</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>v1.1.0; enriched 2026-10-23 with developmental facts from Wolff ch.17 (Development of the Human Eye, pp.646-655, uploaded file 16.pdf) - each fact page-referenced; validate 18/18, pytest 10+14 green</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add SCL-001..004 rows to extraction tracker
</commit_message>
<xml_diff>
--- a/Anatomy_Extraction_Master_Tracker_v2.xlsx
+++ b/Anatomy_Extraction_Master_Tracker_v2.xlsx
@@ -1052,7 +1052,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U19"/>
+  <dimension ref="A1:U23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="5"/>
   <sheetData>
     <row r="1">
@@ -3045,6 +3045,434 @@
       <c r="U19" t="inlineStr">
         <is>
           <t>v1.1.0; enriched 2026-10-23 with developmental facts from Wolff ch.17 (Development of the Human Eye, pp.646-655, uploaded file 16.pdf) - each fact page-referenced; validate 18/18, pytest 10+14 green</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>SCL-001</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Sclera</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Sclera (Proper)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>15,17</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>ch7: 269-278 (episclera 270-271, dimensions 272, apertures 272-274, organization 275-276, blood/nerve 276-277, ageing 277-278)</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>sclera.json</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff scan 7777.pdf)</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 22/22, 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>v1.0.0; created 2026-10-23 from Wolff Ch.7 pp.269-278</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>SCL-002</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Sclera</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Episclera</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>ch7: 270-271, 277; ch8: 280</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>episclera.json</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff scans 7777+8888)</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 22/22, 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>v1.0.0; ciliary injection, sub-Tenon plane, episcleritis</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>SCL-003</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Sclera</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Lamina Cribrosa</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>15,17</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>ch7: 272-274; ch15: 497; ch17: 631</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>lamina-cribrosa.json</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff scans 7777+13+16)</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 22/22, 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>v1.0.0; glaucomatous cupping; primitive PLC at 14 weeks</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>SCL-004</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Sclera</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Scleral Spur</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>7,17</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>ch8: 284, 280; ch7: 275; ch17: 632-633</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>scleral-spur.json</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff scans 8888+7777+16)</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 22/22, 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>v1.0.0; SSC myofibroblasts; miotic mechanism; gonioscopic landmark</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Enrich 4 sclera cards with Wolff development facts from 16.pdf (v1.1.0): collagen maturation, lamina cribrosa 11-21 wks, spur 4mo, vascular plexuses 12wks, IGF-II/myopia growth regulation + tracker notes
</commit_message>
<xml_diff>
--- a/Anatomy_Extraction_Master_Tracker_v2.xlsx
+++ b/Anatomy_Extraction_Master_Tracker_v2.xlsx
@@ -3081,7 +3081,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>ch7: 269-278 (episclera 270-271, dimensions 272, apertures 272-274, organization 275-276, blood/nerve 276-277, ageing 277-278)</t>
+          <t>ch7: 269-278 (episclera 270-271, dimensions 272, apertures 272-274, organization 275-276, blood/nerve 276-277, ageing 277-278) | ch17: 628-632 (17.3 SCLERA opening: neural crest origin, &lt;6.5 wks 8-9 layers, demarcation mid-7th wk 15 layers, 9th wk 48nm, 30-&gt;50 layers, IGF-II/myopia) [16.pdf + full-book scan]</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -3151,7 +3151,7 @@
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>v1.0.0; created 2026-10-23 from Wolff Ch.7 pp.269-278</t>
+          <t>v1.0.0; created 2026-10-23 from Wolff Ch.7 pp.269-278 | v1.1.0+v1.2.0 dev enrichment 2026-10-23</t>
         </is>
       </c>
     </row>
@@ -3188,7 +3188,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>ch7: 270-271, 277; ch8: 280</t>
+          <t>ch7: 270-271, 277; ch8: 280 | ch17: 632 (development: deep/intrascleral plexuses + aqueous veins first recognizable ~12 wks) [16.pdf]</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>v1.0.0; ciliary injection, sub-Tenon plane, episcleritis</t>
+          <t>v1.0.0; ciliary injection, sub-Tenon plane, episcleritis | v1.1.0 dev enrichment 2026-10-23</t>
         </is>
       </c>
     </row>
@@ -3295,7 +3295,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>ch7: 272-274; ch15: 497; ch17: 631</t>
+          <t>ch7: 272-274; ch15: 497; ch17: 631 | ch17: 631 (development: mesenchymal cells transverse between nerve fibres ~11-12 wks; PLC 12 wks; defined 21 wks, Rhodes 1978) [16.pdf]</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -3365,7 +3365,7 @@
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>v1.0.0; glaucomatous cupping; primitive PLC at 14 weeks</t>
+          <t>v1.0.0; glaucomatous cupping; primitive PLC at 14 weeks | v1.1.0 dev enrichment 2026-10-23</t>
         </is>
       </c>
     </row>
@@ -3402,7 +3402,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>ch8: 284, 280; ch7: 275; ch17: 632-633</t>
+          <t>ch8: 284, 280; ch7: 275; ch17: 632-633 | ch17: 632 (development: spur appears ~4 mo/70mm at inner limbus; ciliary insertion mid-7th mo; circular collagen) [16.pdf]</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -3472,7 +3472,7 @@
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>v1.0.0; SSC myofibroblasts; miotic mechanism; gonioscopic landmark</t>
+          <t>v1.0.0; SSC myofibroblasts; miotic mechanism; gonioscopic landmark | v1.1.0 dev enrichment 2026-10-23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Enrich 5 cornea cards with Wolff 17.2 CORNEA development facts (v1.1.x/v1.2.x): stroma primary/secondary waves + keratan sulphate 6mo + diameter growth 2-9.3mm, endothelium first neural-crest wave, epithelium surface maturation, Descemet membrane-units 30-40 layers at birth, Bowman late 4th month keratocyte account (printed pp.624-628, full-book scan تتت.pdf) + tracker COR rows
</commit_message>
<xml_diff>
--- a/Anatomy_Extraction_Master_Tracker_v2.xlsx
+++ b/Anatomy_Extraction_Master_Tracker_v2.xlsx
@@ -1195,7 +1195,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>ch7: 235-267; ch2: 51-65, 82; ch6: 216-221; ch17: 624-628</t>
+          <t>ch7: 235-267; ch2: 51-65, 82; ch6: 216-221; ch17: 624-628 | ch17: 624, 625 (17.2: lens vesicle separation 33 d; surface maturation: 7th wk 10-20 um pentagonal/hexagonal + glycogen; 2nd-3rd mo 15-20 um; 4th mo 3 cell types; adult surface at eyelid opening 5-6 mo) [full-book scan تتت.pdf]</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1260,7 +1260,7 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Filename fixed to match repo (corneal-epithelium.json); supporting material from ch2 (limbus/conjunctiva), ch6 (dimensions, stem cells) and ch17 (development) in addition to ch7; pages 233-234 and 259-265 of ch7 not yet provided - definition supported by ch6 p.216; revalidated 2026-10-17 after bilingual keyword surface + alias (v1.0.1)</t>
+          <t>Filename fixed to match repo (corneal-epithelium.json); supporting material from ch2 (limbus/conjunctiva), ch6 (dimensions, stem cells) and ch17 (development) in addition to ch7; pages 233-234 and 259-265 of ch7 not yet provided - definition supported by ch6 p.216; revalidated 2026-10-17 after bilingual keyword surface + alias (v1.0.1) | v1.2.0 dev enrichment 2026-10-24: epithelial surface maturation timeline appended to histology</t>
         </is>
       </c>
     </row>
@@ -1297,7 +1297,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>ch7: 247-249; ch17: 627-628</t>
+          <t>ch7: 247-249; ch17: 627-628 | ch17: 627, 628 (17.2 BOWMAN'S ZONE: not formed until late 4th mo; always acellular; superficial keratocytes presumed source; anchoring filaments 474nm x 17.6nm at 17-18 wks, adult at 26 wks, intermingled at birth, dense collagen at 1 yr, Fig 17.13) [full-book scan تتت.pdf]</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1362,7 +1362,7 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Extracted from already-read pages: ch7 247-249 (structure) + ch17 627-628 (development, synthesised by basal epithelial cells). 8/8 fields documented with page sources; statpearls only for avascular statements. Awaiting user PR.</t>
+          <t>Extracted from already-read pages: ch7 247-249 (structure) + ch17 627-628 (development, synthesised by basal epithelial cells). 8/8 fields documented with page sources; statpearls only for avascular statements. Awaiting user PR. | v1.1.0 dev enrichment 2026-10-24: developmental timing + keratocyte account + anchoring-filament maturation appended to histology</t>
         </is>
       </c>
     </row>
@@ -1399,7 +1399,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>ch7: 249-252, 266, 268-270; ch6: 216-218</t>
+          <t>ch7: 249-252, 266, 268-270; ch6: 216-218 | ch17: 624-626, 628 (17.2 PRIMARY CORNEAL STROMA + STROMA: trigger at 33 d; primary stroma fine filaments; HA swelling; 3 waves Fig 17.9; keratocytes type I collagen secondary stroma; double width then dehydration; GAG before collagen; keratan sulphate 6 mo; interstitial+appositional lamellar growth; 8 wk 5-8 rows; 35 mm 15 layers; diameter 2-&gt;9.3 mm 12-35 wks, Ehlers 1968) [full-book scan تتت.pdf]</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>Extracted from already-read pages: ch7 249-252 (structure), 266 (transparency), 268-270 (limbal transition, ground substance) + ch6 216-218 (dimensions). Richest card (~970 tokens). 8/8 fields documented. Awaiting user PR.</t>
+          <t>Extracted from already-read pages: ch7 249-252 (structure), 266 (transparency), 268-270 (limbal transition, ground substance) + ch6 216-218 (dimensions). Richest card (~970 tokens). 8/8 fields documented. Awaiting user PR. | v1.1.0 dev enrichment 2026-10-24: full development narrative appended to histology</t>
         </is>
       </c>
     </row>
@@ -1501,7 +1501,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>ch7: 251-258; ch17: 626; ch8: 284, 286</t>
+          <t>ch7: 251-258; ch17: 626; ch8: 284, 286 | ch17: 627 (17.2 DESCEMET'S MEMBRANE AND ENDOTHELIUM: membrane-units 1 layer @12 wks, ~10 @6th mo, 30-40 @birth; cross-link filaments 170x40 nm; last-trimester compaction; hexagonal triangle pattern ~110 nm; banded zone max 3 um at birth; non-banded zone thickens with age, Murphy 1984/Tripathi 1984) [full-book scan تتت.pdf]</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1566,7 +1566,7 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>Extracted from already-read pages: ch7 251-255 (membrane), 256-257 (endothelial attachment) + ch17 626 (development) + ch8 284/286 (Schwalbe/angle). 8/8 fields documented; innervation = not_available (posterior stromal nerves end before reaching it, ch7 p.267). Awaiting user PR.</t>
+          <t>Extracted from already-read pages: ch7 251-255 (membrane), 256-257 (endothelial attachment) + ch17 626 (development) + ch8 284/286 (Schwalbe/angle). 8/8 fields documented; innervation = not_available (posterior stromal nerves end before reaching it, ch7 p.267). Awaiting user PR. | v1.1.0 dev enrichment 2026-10-24: membrane-units mechanism + banded-zone ultrastructure appended to histology</t>
         </is>
       </c>
     </row>
@@ -1603,7 +1603,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>ch7: 233-263; ch8: 284, 286</t>
+          <t>ch7: 233-263; ch8: 284, 286 | ch17: 625-627 (17.2: first wave of neural crest from optic-cup rim beneath epithelial basal lamina -&gt; primordial endothelium, Tripathi 1974; double layer @40 d Fig 17.10; single layer @3rd mo/63 mm; apical zonulae occludentes mid-4th mo with onset of aqueous production) [full-book scan تتت.pdf]</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>Filename fixed to match repo (corneal-endothelium.json). Reference registry corrected: authors are Bron, Tripathi &amp; Tripathi, Chapman &amp; Hall Medical, 8th ed., 1997 (verified vs title/copyright pages). innervation field = not_available, re-check ch.7.1 during full-text extraction.; keywords v1.1.1 (Arabic + cell density/deturgescence), revalidated 2026-10-17; pages 259-265 still outstanding - nerves pages 266-267 (read) support the posterior-stroma-only innervation pattern</t>
+          <t>Filename fixed to match repo (corneal-endothelium.json). Reference registry corrected: authors are Bron, Tripathi &amp; Tripathi, Chapman &amp; Hall Medical, 8th ed., 1997 (verified vs title/copyright pages). innervation field = not_available, re-check ch.7.1 during full-text extraction.; keywords v1.1.1 (Arabic + cell density/deturgescence), revalidated 2026-10-17; pages 259-265 still outstanding - nerves pages 266-267 (read) support the posterior-stroma-only innervation pattern | v1.2.0 dev enrichment 2026-10-24: neural-crest origin + layering timeline appended to histology</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add OpticNerve knowledge cards (ON-001..005, Wolff Ch.15 'The Visual Pathway' printed pp.495-534): whole nerve (1M axons, 800-1200 fascicles, myelination doubles diameter 1.5-3.0mm, segments+relations), optic disc (disc/cup/rim metrics Table 15.1, zones alpha/beta, ONH watershed supply), sheaths (dura 0.35-0.5mm/arachnoid 10um/pia-glia), septa (4th-month invasion, 6-9 primary, glial septum & decussation), blood supply (pial network, Zinn-Haller, venous drainage, BBB) + tracker ON rows
</commit_message>
<xml_diff>
--- a/Anatomy_Extraction_Master_Tracker_v2.xlsx
+++ b/Anatomy_Extraction_Master_Tracker_v2.xlsx
@@ -1052,7 +1052,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U23"/>
+  <dimension ref="A1:U28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="5"/>
   <sheetData>
     <row r="1">
@@ -3473,6 +3473,541 @@
       <c r="U23" t="inlineStr">
         <is>
           <t>v1.0.0; SSC myofibroblasts; miotic mechanism; gonioscopic landmark | v1.1.0 dev enrichment 2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>ON-001</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Optic Nerve</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Optic Nerve (Whole Nerve)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>ch15: 495-499, 508-509, 515-521, 524 (papillomotor/centrifugal fibres + 800-1200 fascicles (Deyl 1895) + axon estimates Polyak/Oppel/Kupfer 515; axon diameters 0.7-10 um, 92% &lt;1 um, microtubules 20-25 nm (Anderson &amp; Hoyt 1969) 521/515; retrolaminar myelination doubles diameter 1.5-&gt;3.0 mm (Minckler 1976) 499; orbit relations incl. ciliary ganglion + CRA entry ~12 mm behind eye 508; scleral canal 0.5 mm 505; orbital length 3 cm 524) [scans 13.pdf+14.pdf]</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>optic-nerve.json</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Done (manual, scans 13.pdf + 14.pdf)</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 27/27, 2026-10-24)</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)]</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>ON-002</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Optic Nerve</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Optic Disc (Optic Nerve Head)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>ch15: 503-508, 528-534 (disc area 0.86-5.54 mm2 mean 2.69±0.7 + macrodiscs &gt;4.09/microdiscs &lt;1.29 (Jonas/Gusek/Naumann 1988, 1991) + Table 15.1 full metrics 505; lamina area 2.88±0.84 mm2 + pore count 227±36 (Jonas 1991) + cup metrics + rim broadest inferior-&gt;superior-&gt;nasal-&gt;temporal, narrowest temporal horizontal in 99.2% 506; cup/disc ratio median 0.3, vertical lower in 93.2%, asymmetry &gt;0.2 diagnostic; parapapillary zones alpha 84.4%/beta 15.2% + POAG alpha 0.65/beta 0.79 507; RNFL visibility order + axon loss 4-5000/yr 508; ONH watershed + zonal arterial supply + venous drainage + opticociliary veins 528-534) [scans 13.pdf+14.pdf]</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>optic-disc.json</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Done (manual, scans 13.pdf + 14.pdf)</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 27/27, 2026-10-24)</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)]</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>ON-003</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Optic Nerve</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Optic Nerve Sheaths</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>ch15: 508-516, 518 (cranial dura splits into periorbita + dural sheath at optic foramen; subdural space potential/artefact 510; dura 0.35-0.5 mm, circular internal + longitudinal/oblique peripheral fibres, collagen 600-700 um as printed, 2-5 outer lamellae 510-511; arachnoid ~10 um, meningothelial multilaminar + trabeculae + corpora amylacea, ends at lamina cribrosa 512; pia-glia / glial mantle of Fuchs + septa + vessels between longitudinal and circular fibres 513; SAS scleral cul-de-sac behind lamina cribrosa, widest anteriorly, wider nasally 515) [scans 13.pdf]</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>optic-nerve-sheath.json</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Done (manual, scans 13.pdf + 14.pdf)</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 27/27, 2026-10-24)</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)]</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>ON-004</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Optic Nerve</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Septa of the Optic Nerve</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>ch15: 499, 515-518, 521 (septa invade with vessels ~4th month; 6-9 primary septa into sectors + dichotomous secondary septa; interseptal spaces rounded in human vs polygonal in other mammals 517; septa = tubes around fascicles, fenestrated; trabecula central vessel with muscular/elastic layers; astrocyte feet + basal lamina + invaginations 120-150 um (Anderson &amp; Hoyt 1969); astrocytes abut capillaries directly in chiasma 521; triangular glial septum separates ventromedial (crossing) from dorsolateral, marks start of decussation 518; support deficiency superior/inferior -&gt; early glaucomatous bowing (Quigley) 499) [scans 13.pdf]</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>optic-nerve-septa.json</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Done (manual, scans 13.pdf + 14.pdf)</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 27/27, 2026-10-24)</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)]</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>ON-005</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Optic Nerve</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Blood Supply of the Optic Nerve</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>ch15: 521-524, 527-534 (pial network double system + septal distribution exact = vessels 521; perichiasmal artery largest intracranial supply, origin superior hypophyseal (Hayreh 1963/Steele &amp; Blunt 1956) vs Dawson 1958 ophthalmic 522; intracanalicular OA sole supply, poor pial network vulnerable to shearing in skull fracture 524; intraorbital: CRA enters 5-15.5 mm behind globe, proximal centripetal vs distal axial, 3 sources, direct branches reach pia in 75% when OA crosses above (82-85% of cases) 524; venous drainage: pial veins + central retinal vein(s) (embryonic 2 channels beside hyaloid artery 3rd month; exit same aspect in 42%, vein anterior to artery in 81% (Fry 1930); intravaginal course 3.8-8 mm) + posterior central vein 527; cavernous sinus blockage does not block CRV flow 528; laminar circle of Zinn (1755)/Haller (1754) branches 1-4 + interfacial precapillaries vulnerable to raised IOP -&gt; disc haemorrhages (Ruskell 1984) 531; prelaminar scleral SPCA vs recurrent choroidal (only 10% choroidal origin, Lieberman 1976) + microvascular cuff 534; SNFL 5 supplies with CRA major 534; BBB incomplete at ONH (pars choroidalis) 534) [scans 13.pdf+14.pdf]</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>optic-nerve-blood-supply.json</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Done (manual, scans 13.pdf + 14.pdf)</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 27/27, 2026-10-24)</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Optic Nerve cards v1.1.0: batch-3 enrichment (printed 525, 535-545, 586-590)
- optic-nerve: proximal-nerve fibre topography + knee of Wilbrand (540-541)
- optic-nerve-blood-supply: orbital pial plexus/CRA course & Hayreh stats (525-526),
  CRA wall structure + GCA rule (526), Zinn-Haller frequency/form/position (530-533),
  chiasmal dorsal/ventral supply Wollschlaeger (541-543)
- optic-disc: Zinn-Haller dispute + positions (530,533), Kuhnt glial gasket (535),
  incomplete ONH BBB + optic pits/papilloedema (534-535)
- optic-nerve-sheath: CRA dural piercing/intravaginal course, CRV dural residence (525-527)
- optic-nerve-septa: intraseptal microvasculature polygonal units (525,529)
- tracker: ON-001..005 col G/U updated
- validate 27/27, pytest 10+14 green
</commit_message>
<xml_diff>
--- a/Anatomy_Extraction_Master_Tracker_v2.xlsx
+++ b/Anatomy_Extraction_Master_Tracker_v2.xlsx
@@ -3509,7 +3509,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>ch15: 495-499, 508-509, 515-521, 524 (papillomotor/centrifugal fibres + 800-1200 fascicles (Deyl 1895) + axon estimates Polyak/Oppel/Kupfer 515; axon diameters 0.7-10 um, 92% &lt;1 um, microtubules 20-25 nm (Anderson &amp; Hoyt 1969) 521/515; retrolaminar myelination doubles diameter 1.5-&gt;3.0 mm (Minckler 1976) 499; orbit relations incl. ciliary ganglion + CRA entry ~12 mm behind eye 508; scleral canal 0.5 mm 505; orbital length 3 cm 524) [scans 13.pdf+14.pdf]</t>
+          <t>ch15: 495-499, 508-509, 515-521, 524 (papillomotor/centrifugal fibres + 800-1200 fascicles (Deyl 1895) + axon estimates Polyak/Oppel/Kupfer 515; axon diameters 0.7-10 um, 92% &lt;1 um, microtubules 20-25 nm (Anderson &amp; Hoyt 1969) 521/515; retrolaminar myelination doubles diameter 1.5-&gt;3.0 mm (Minckler 1976) 499; orbit relations incl. ciliary ganglion + CRA entry ~12 mm behind eye 508; scleral canal 0.5 mm 505; orbital length 3 cm 524) [scans 13.pdf+14.pdf] | v1.1.0 pages: 540-541 + 530-560.pdf/586.pdf</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -3579,7 +3579,7 @@
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)]</t>
+          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)] | v1.1.0 enrichment 2026-10-24: batch-3 pages (printed 525, 535-545, 586-590 from scans 530-560.pdf = printed 525-550 verified 1:1 + 586.pdf = printed 586-590 verified 1:1) read visually and mined; fibre topography of the proximal nerve appended to histology (crossed/uncrossed separation begins proximally with crossing fibres medial to the pial septum end; nasal fibres form a quadrilateral sheet; inferior nasal fibres loop forward into the contralateral proximal nerve up to 3 mm = knee of Wilbrand) + clinical consequence (proximal nerve compression affects both eyes' fields; pituitary chiasmal involvement heralded by upper bitemporal quadrantanopia, pp.540-541); bilingual keywords extended; validate 27/27 + pytest 10+14 green</t>
         </is>
       </c>
     </row>
@@ -3616,7 +3616,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>ch15: 503-508, 528-534 (disc area 0.86-5.54 mm2 mean 2.69±0.7 + macrodiscs &gt;4.09/microdiscs &lt;1.29 (Jonas/Gusek/Naumann 1988, 1991) + Table 15.1 full metrics 505; lamina area 2.88±0.84 mm2 + pore count 227±36 (Jonas 1991) + cup metrics + rim broadest inferior-&gt;superior-&gt;nasal-&gt;temporal, narrowest temporal horizontal in 99.2% 506; cup/disc ratio median 0.3, vertical lower in 93.2%, asymmetry &gt;0.2 diagnostic; parapapillary zones alpha 84.4%/beta 15.2% + POAG alpha 0.65/beta 0.79 507; RNFL visibility order + axon loss 4-5000/yr 508; ONH watershed + zonal arterial supply + venous drainage + opticociliary veins 528-534) [scans 13.pdf+14.pdf]</t>
+          <t>ch15: 503-508, 528-534 (disc area 0.86-5.54 mm2 mean 2.69±0.7 + macrodiscs &gt;4.09/microdiscs &lt;1.29 (Jonas/Gusek/Naumann 1988, 1991) + Table 15.1 full metrics 505; lamina area 2.88±0.84 mm2 + pore count 227±36 (Jonas 1991) + cup metrics + rim broadest inferior-&gt;superior-&gt;nasal-&gt;temporal, narrowest temporal horizontal in 99.2% 506; cup/disc ratio median 0.3, vertical lower in 93.2%, asymmetry &gt;0.2 diagnostic; parapapillary zones alpha 84.4%/beta 15.2% + POAG alpha 0.65/beta 0.79 507; RNFL visibility order + axon loss 4-5000/yr 508; ONH watershed + zonal arterial supply + venous drainage + opticociliary veins 528-534) [scans 13.pdf+14.pdf] | v1.1.0 pages: 530, 533, 534-535 + 530-560.pdf/586.pdf</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -3686,7 +3686,7 @@
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)]</t>
+          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)] | v1.1.0 enrichment 2026-10-24: from batch-3 pages (525, 535-545, 586-590): circle of Zinn-Haller frequency dispute (Olver 1990 frequently present vs Hayreh small proportion; often incomplete Levitzky &amp; Henkind 1969; ABSENT in sub-human primates Hayreh 1964; horizontal-ellipse intrascleral anastomosis of medial+lateral paraoptic SPCA branches; paraoptic replacements when absent) + positional variants (apposed/distant/anterior intrascleral/posterior extrascleral; axial position on SEM) appended to blood_supply; marginal tissue of Kuhnt glial 'gasket' tight junctions appended to histology (Tso/Shih/McLean 1975); incomplete ONH blood-brain barrier with HRP tracer route choroid-&gt;prelaminar-&gt;lamina septa-&gt;retrolaminar + implications for optic pits and papilloedema appended to clinical (pp.534-535); bilingual keywords extended; validate 27/27 + pytest 10+14 green</t>
         </is>
       </c>
     </row>
@@ -3723,7 +3723,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>ch15: 508-516, 518 (cranial dura splits into periorbita + dural sheath at optic foramen; subdural space potential/artefact 510; dura 0.35-0.5 mm, circular internal + longitudinal/oblique peripheral fibres, collagen 600-700 um as printed, 2-5 outer lamellae 510-511; arachnoid ~10 um, meningothelial multilaminar + trabeculae + corpora amylacea, ends at lamina cribrosa 512; pia-glia / glial mantle of Fuchs + septa + vessels between longitudinal and circular fibres 513; SAS scleral cul-de-sac behind lamina cribrosa, widest anteriorly, wider nasally 515) [scans 13.pdf]</t>
+          <t>ch15: 508-516, 518 (cranial dura splits into periorbita + dural sheath at optic foramen; subdural space potential/artefact 510; dura 0.35-0.5 mm, circular internal + longitudinal/oblique peripheral fibres, collagen 600-700 um as printed, 2-5 outer lamellae 510-511; arachnoid ~10 um, meningothelial multilaminar + trabeculae + corpora amylacea, ends at lamina cribrosa 512; pia-glia / glial mantle of Fuchs + septa + vessels between longitudinal and circular fibres 513; SAS scleral cul-de-sac behind lamina cribrosa, widest anteriorly, wider nasally 515) [scans 13.pdf] | v1.1.0 pages: 525-527 + 530-560.pdf/586.pdf</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -3793,7 +3793,7 @@
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)]</t>
+          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)] | v1.1.0 enrichment 2026-10-24: from batch-3 pages: CRA-sheath relationships appended to blood_supply (CRA pierces dura 5-15.5 mm behind globe inferomedially; intravaginal course 0.9-2.5 mm mainly within the subarachnoid space; vertical nerve entry with right-angled bend; intravaginal pial branches near the arterial entry; intraorbital branches supply pia from globe to canal in half the nerves) + CRV intravaginal course longer than the artery (3.8-8 mm) with greater dural residence appended to venous_drainage (pp.525-527); bilingual keywords extended; validate 27/27 + pytest 10+14 green</t>
         </is>
       </c>
     </row>
@@ -3830,7 +3830,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>ch15: 499, 515-518, 521 (septa invade with vessels ~4th month; 6-9 primary septa into sectors + dichotomous secondary septa; interseptal spaces rounded in human vs polygonal in other mammals 517; septa = tubes around fascicles, fenestrated; trabecula central vessel with muscular/elastic layers; astrocyte feet + basal lamina + invaginations 120-150 um (Anderson &amp; Hoyt 1969); astrocytes abut capillaries directly in chiasma 521; triangular glial septum separates ventromedial (crossing) from dorsolateral, marks start of decussation 518; support deficiency superior/inferior -&gt; early glaucomatous bowing (Quigley) 499) [scans 13.pdf]</t>
+          <t>ch15: 499, 515-518, 521 (septa invade with vessels ~4th month; 6-9 primary septa into sectors + dichotomous secondary septa; interseptal spaces rounded in human vs polygonal in other mammals 517; septa = tubes around fascicles, fenestrated; trabecula central vessel with muscular/elastic layers; astrocyte feet + basal lamina + invaginations 120-150 um (Anderson &amp; Hoyt 1969); astrocytes abut capillaries directly in chiasma 521; triangular glial septum separates ventromedial (crossing) from dorsolateral, marks start of decussation 518; support deficiency superior/inferior -&gt; early glaucomatous bowing (Quigley) 499) [scans 13.pdf] | v1.1.0 pages: 525, 529 + 530-560.pdf/586.pdf</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -3900,7 +3900,7 @@
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)]</t>
+          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)] | v1.1.0 enrichment 2026-10-24: from batch-3 pages: pial plexus centripetal branches each within a glial-coated connective-tissue core (p.525) + CRA intraneural branches anastomosing with the septal arteriolar/capillary system (p.529) + full intraseptal microvasculature account (large precapillaries/capillaries confined to septae in transverse and longitudinal polygonal units; extensive anastomosis, size non-uniformity, numbers increasing near posterior laminal bowing; anterior anastomosis with laminar vessels, posterior with intraorbital septal system — Lieberman/Maumenee/Green 1976) appended to blood_supply; bilingual keywords extended; validate 27/27 + pytest 10+14 green</t>
         </is>
       </c>
     </row>
@@ -3937,7 +3937,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>ch15: 521-524, 527-534 (pial network double system + septal distribution exact = vessels 521; perichiasmal artery largest intracranial supply, origin superior hypophyseal (Hayreh 1963/Steele &amp; Blunt 1956) vs Dawson 1958 ophthalmic 522; intracanalicular OA sole supply, poor pial network vulnerable to shearing in skull fracture 524; intraorbital: CRA enters 5-15.5 mm behind globe, proximal centripetal vs distal axial, 3 sources, direct branches reach pia in 75% when OA crosses above (82-85% of cases) 524; venous drainage: pial veins + central retinal vein(s) (embryonic 2 channels beside hyaloid artery 3rd month; exit same aspect in 42%, vein anterior to artery in 81% (Fry 1930); intravaginal course 3.8-8 mm) + posterior central vein 527; cavernous sinus blockage does not block CRV flow 528; laminar circle of Zinn (1755)/Haller (1754) branches 1-4 + interfacial precapillaries vulnerable to raised IOP -&gt; disc haemorrhages (Ruskell 1984) 531; prelaminar scleral SPCA vs recurrent choroidal (only 10% choroidal origin, Lieberman 1976) + microvascular cuff 534; SNFL 5 supplies with CRA major 534; BBB incomplete at ONH (pars choroidalis) 534) [scans 13.pdf+14.pdf]</t>
+          <t>ch15: 521-524, 527-534 (pial network double system + septal distribution exact = vessels 521; perichiasmal artery largest intracranial supply, origin superior hypophyseal (Hayreh 1963/Steele &amp; Blunt 1956) vs Dawson 1958 ophthalmic 522; intracanalicular OA sole supply, poor pial network vulnerable to shearing in skull fracture 524; intraorbital: CRA enters 5-15.5 mm behind globe, proximal centripetal vs distal axial, 3 sources, direct branches reach pia in 75% when OA crosses above (82-85% of cases) 524; venous drainage: pial veins + central retinal vein(s) (embryonic 2 channels beside hyaloid artery 3rd month; exit same aspect in 42%, vein anterior to artery in 81% (Fry 1930); intravaginal course 3.8-8 mm) + posterior central vein 527; cavernous sinus blockage does not block CRV flow 528; laminar circle of Zinn (1755)/Haller (1754) branches 1-4 + interfacial precapillaries vulnerable to raised IOP -&gt; disc haemorrhages (Ruskell 1984) 531; prelaminar scleral SPCA vs recurrent choroidal (only 10% choroidal origin, Lieberman 1976) + microvascular cuff 534; SNFL 5 supplies with CRA major 534; BBB incomplete at ONH (pars choroidalis) 534) [scans 13.pdf+14.pdf] | v1.1.0 pages: 525-526, 530, 533, 541, 543 + 530-560.pdf/586.pdf</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -4007,7 +4007,7 @@
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)]</t>
+          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)] | v1.1.0 enrichment 2026-10-24: batch-3 pages mined heavily: intraorbital layers block extended with the long-awaited p.525 material (pial plexus tortuous anastomoses reinforced at nerve-globe junction by scleral SPCA/circle of Zinn; centripetal branches within glial-coated cores; CRA origin variants relative to ophthalmic artery crossing; CRA course - dura piercing 5-15.5 mm inferomedially, intravaginal 0.9-2.5 mm in subarachnoid space, vertical entry + right-angled bend, ~5/3/8 intraorbital/intravaginal/intraneural branches; Hayreh 1963 stats - branches in all but 3.1%, none to lamina cribrosa, lacking intraorbital 47.8%/intravaginal 5.3%/intraneural 25%; collaterals superior/inferior per OA crossing, lateral rare vs Hughes 1954; CRA pial territory always inferior, superior least) + blood_supply extended with CRA wall structure (intima duplicated BM thickening with age; IEL irregular, disappears at lamina, absent from retinal arteries; media ~6 layers; adventitia continuous with septa) + GCA rule (only IEL-bearing vessels affected; retinal arteries spared - Cogan 1974) + Zinn-Haller frequency/form/position (pp.530-533) + chiasmal arterial supply (rich collateral anastomosis; Wollschlaeger 1971 630 specimens dorsal A1/ventral ICA-ACOMM with A2 contribution always per Perlmutter &amp; Rhoton 1976, no PCOMM/PCA/basilar contributions, superior hypophyseal + MCA feeders, dorsal/ventral classification) (pp.541-543) + GCA fact added to clinical; bilingual keywords extended; validate 27/27 + pytest 10+14 green</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update optic nerve knowledge cards and tracker
</commit_message>
<xml_diff>
--- a/Anatomy_Extraction_Master_Tracker_v2.xlsx
+++ b/Anatomy_Extraction_Master_Tracker_v2.xlsx
@@ -3509,7 +3509,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>ch15: 495-499, 508-509, 515-521, 524 (papillomotor/centrifugal fibres + 800-1200 fascicles (Deyl 1895) + axon estimates Polyak/Oppel/Kupfer 515; axon diameters 0.7-10 um, 92% &lt;1 um, microtubules 20-25 nm (Anderson &amp; Hoyt 1969) 521/515; retrolaminar myelination doubles diameter 1.5-&gt;3.0 mm (Minckler 1976) 499; orbit relations incl. ciliary ganglion + CRA entry ~12 mm behind eye 508; scleral canal 0.5 mm 505; orbital length 3 cm 524) [scans 13.pdf+14.pdf] | v1.1.0 pages: 540-541 + 530-560.pdf/586.pdf</t>
+          <t>ch15: 495-499, 508-509, 515-521, 524 (papillomotor/centrifugal fibres + 800-1200 fascicles (Deyl 1895) + axon estimates Polyak/Oppel/Kupfer 515; axon diameters 0.7-10 um, 92% &lt;1 um, microtubules 20-25 nm (Anderson &amp; Hoyt 1969) 521/515; retrolaminar myelination doubles diameter 1.5-&gt;3.0 mm (Minckler 1976) 499; orbit relations incl. ciliary ganglion + CRA entry ~12 mm behind eye 508; scleral canal 0.5 mm 505; orbital length 3 cm 524) [scans 13.pdf+14.pdf] | v1.1.0 pages: 540-541 + 530-560.pdf/586.pdf; ch1: 23, 24, 25, 26 (bony optic canal between two roots of lesser wing; chiasmal sulcus rarely contacting chiasm; jugum sphenoidale; anterior/middle clinoid + caroticoclinoid foramen; cavernous sinus extent &amp; intercavernous connections; diaphragma sellae; SOF vs optic canal); ch5: 190 (cavernous lateral wall: III/IV/V1/V2, VI free inferolateral to ICA) | v1.3.0 sources: StatPearls NBK507907 (CN II, 2022) + NBK542287 (Optic Chiasm, 2023) read in full</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -3579,7 +3579,7 @@
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)] | v1.1.0 enrichment 2026-10-24: batch-3 pages (printed 525, 535-545, 586-590 from scans 530-560.pdf = printed 525-550 verified 1:1 + 586.pdf = printed 586-590 verified 1:1) read visually and mined; fibre topography of the proximal nerve appended to histology (crossed/uncrossed separation begins proximally with crossing fibres medial to the pial septum end; nasal fibres form a quadrilateral sheet; inferior nasal fibres loop forward into the contralateral proximal nerve up to 3 mm = knee of Wilbrand) + clinical consequence (proximal nerve compression affects both eyes' fields; pituitary chiasmal involvement heralded by upper bitemporal quadrantanopia, pp.540-541); bilingual keywords extended; validate 27/27 + pytest 10+14 green</t>
+          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)] | v1.1.0 enrichment 2026-10-24: batch-3 pages (printed 525, 535-545, 586-590 from scans 530-560.pdf = printed 525-550 verified 1:1 + 586.pdf = printed 586-590 verified 1:1) read visually and mined; fibre topography of the proximal nerve appended to histology (crossed/uncrossed separation begins proximally with crossing fibres medial to the pial septum end; nasal fibres form a quadrilateral sheet; inferior nasal fibres loop forward into the contralateral proximal nerve up to 3 mm = knee of Wilbrand) + clinical consequence (proximal nerve compression affects both eyes' fields; pituitary chiasmal involvement heralded by upper bitemporal quadrantanopia, pp.540-541); bilingual keywords extended; validate 27/27 + pytest 10+14 green | v1.2.0 (2026-10-26) batch-4: skull-base relations &amp; cavernous sinus topography from owner-supplied text (printed 23-26, 190) - bony canal (two roots of lesser wing, direction forwards/laterally/downwards), chiasmal sulcus above/behind -&gt; chiasm elevation by sellar expansion, anterior clinoid + caroticoclinoid foramen, cavernous sinus extent pp.23-26; localization contrast: CN II outside sinus whose lateral wall carries III/IV/V1/V2 with VI free (p.190) -&gt; vision spared in cavernous lesions; pages 22, 27-29, 189, 191, 282, 359-360 screened: no optic-nerve facts, not cited; bilingual keywords +20; validate 27/27 + pytest 10+14 green | v1.3.0 (2026-10-26) StatPearls round: both articles fetched via /sites/books/ and read in FULL (2,597 + 5,014 words) with 25/25 literal quote checks passed before writing. definition: explicit synaptic targets (SCN circadian, LGN, pretectal, superior colliculus) + afferent limb of light and accommodation reflexes; location: chiasm ~10 mm above pituitary in suprasellar cistern, adjacent to third-ventricle anterior wall/floor junction; clinical: chiasm position variants (normo-fixed 85% / pre-fixed 7.5% / post-fixed 8%, cadaver study) + lesion localisation (pre-chiasmal ipsilateral monocular; pituitary macroadenoma compresses inferior chiasm -&gt; superior temporal loss before bitemporal; optic pathway glioma 3-5% paediatric / 6.6-20% NF1) + RAPD/Marcus Gunn with swinging flashlight test; histology: unmyelinated-until-lamina rationale (retinal light path), optic stalk 4th week -&gt; nerve, hyaloid vessels -&gt; CRA/CRV, myelination timeline (LGN 5mo -&gt; tract 6mo -&gt; chiasm 6-7mo -&gt; nerve 8mo; crossed 7-8wk, uncrossed ~11wk) + modern-imaging caveat on knees of Wilbrand (failed identification, shifting rejection in normals, possible sequela of long-term monocular neuropathy). Registry +2 statpearls entries (14 total). validate 27/27 + pytest green.</t>
         </is>
       </c>
     </row>
@@ -3616,7 +3616,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>ch15: 503-508, 528-534 (disc area 0.86-5.54 mm2 mean 2.69±0.7 + macrodiscs &gt;4.09/microdiscs &lt;1.29 (Jonas/Gusek/Naumann 1988, 1991) + Table 15.1 full metrics 505; lamina area 2.88±0.84 mm2 + pore count 227±36 (Jonas 1991) + cup metrics + rim broadest inferior-&gt;superior-&gt;nasal-&gt;temporal, narrowest temporal horizontal in 99.2% 506; cup/disc ratio median 0.3, vertical lower in 93.2%, asymmetry &gt;0.2 diagnostic; parapapillary zones alpha 84.4%/beta 15.2% + POAG alpha 0.65/beta 0.79 507; RNFL visibility order + axon loss 4-5000/yr 508; ONH watershed + zonal arterial supply + venous drainage + opticociliary veins 528-534) [scans 13.pdf+14.pdf] | v1.1.0 pages: 530, 533, 534-535 + 530-560.pdf/586.pdf</t>
+          <t>ch15: 503-508, 528-534 (disc area 0.86-5.54 mm2 mean 2.69±0.7 + macrodiscs &gt;4.09/microdiscs &lt;1.29 (Jonas/Gusek/Naumann 1988, 1991) + Table 15.1 full metrics 505; lamina area 2.88±0.84 mm2 + pore count 227±36 (Jonas 1991) + cup metrics + rim broadest inferior-&gt;superior-&gt;nasal-&gt;temporal, narrowest temporal horizontal in 99.2% 506; cup/disc ratio median 0.3, vertical lower in 93.2%, asymmetry &gt;0.2 diagnostic; parapapillary zones alpha 84.4%/beta 15.2% + POAG alpha 0.65/beta 0.79 507; RNFL visibility order + axon loss 4-5000/yr 508; ONH watershed + zonal arterial supply + venous drainage + opticociliary veins 528-534) [scans 13.pdf+14.pdf] | v1.1.0 pages: 530, 533, 534-535 + 530-560.pdf/586.pdf | v1.2.0 pages: ch15: 494-495 (Anderson 1969 Fig 15.8: prelaminar astrocytic tubes with perpendicular astrocytes + intratubular capillaries; laminar fascicle astrocyte layer + connective-tissue mantle; postlaminar oligodendrocyte columns; border tissue of Jacoby cuff -&gt; intermediary tissue of Kuhnt forwards, glial mantle backwards)</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -3686,7 +3686,7 @@
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)] | v1.1.0 enrichment 2026-10-24: from batch-3 pages (525, 535-545, 586-590): circle of Zinn-Haller frequency dispute (Olver 1990 frequently present vs Hayreh small proportion; often incomplete Levitzky &amp; Henkind 1969; ABSENT in sub-human primates Hayreh 1964; horizontal-ellipse intrascleral anastomosis of medial+lateral paraoptic SPCA branches; paraoptic replacements when absent) + positional variants (apposed/distant/anterior intrascleral/posterior extrascleral; axial position on SEM) appended to blood_supply; marginal tissue of Kuhnt glial 'gasket' tight junctions appended to histology (Tso/Shih/McLean 1975); incomplete ONH blood-brain barrier with HRP tracer route choroid-&gt;prelaminar-&gt;lamina septa-&gt;retrolaminar + implications for optic pits and papilloedema appended to clinical (pp.534-535); bilingual keywords extended; validate 27/27 + pytest 10+14 green</t>
+          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)] | v1.1.0 enrichment 2026-10-24: from batch-3 pages (525, 535-545, 586-590): circle of Zinn-Haller frequency dispute (Olver 1990 frequently present vs Hayreh small proportion; often incomplete Levitzky &amp; Henkind 1969; ABSENT in sub-human primates Hayreh 1964; horizontal-ellipse intrascleral anastomosis of medial+lateral paraoptic SPCA branches; paraoptic replacements when absent) + positional variants (apposed/distant/anterior intrascleral/posterior extrascleral; axial position on SEM) appended to blood_supply; marginal tissue of Kuhnt glial 'gasket' tight junctions appended to histology (Tso/Shih/McLean 1975); incomplete ONH blood-brain barrier with HRP tracer route choroid-&gt;prelaminar-&gt;lamina septa-&gt;retrolaminar + implications for optic pits and papilloedema appended to clinical (pp.534-535); bilingual keywords extended; validate 27/27 + pytest 10+14 green | v1.2.0 (2026-10-26) batch-5: owner text printed 494 (+495 continuation verified visually from scan render) - prelaminar astrocytic-tube architecture (bundles + perpendicular astrocytes, capillaries within tubes), peripheral astrocyte cuff = border tissue of Jacoby continuing forwards as intermediary tissue of Kuhnt and backwards in continuity with glial mantle deep to pia, laminar astrocyte layer + mantle of connective tissue (collagen/elastic/fibroblasts/capillaries) thinner than prelaminar, postlaminar myelination with columns of oligodendrocytes + few astrocytes, glial separation rule (Anderson/Hoyt/Hogan 1967) with CRA-adventitia exception (Ikui 1964) appended to layers[1..3]; keywords +10; validate 27/27 + pytest green.</t>
         </is>
       </c>
     </row>
@@ -3723,7 +3723,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>ch15: 508-516, 518 (cranial dura splits into periorbita + dural sheath at optic foramen; subdural space potential/artefact 510; dura 0.35-0.5 mm, circular internal + longitudinal/oblique peripheral fibres, collagen 600-700 um as printed, 2-5 outer lamellae 510-511; arachnoid ~10 um, meningothelial multilaminar + trabeculae + corpora amylacea, ends at lamina cribrosa 512; pia-glia / glial mantle of Fuchs + septa + vessels between longitudinal and circular fibres 513; SAS scleral cul-de-sac behind lamina cribrosa, widest anteriorly, wider nasally 515) [scans 13.pdf] | v1.1.0 pages: 525-527 + 530-560.pdf/586.pdf</t>
+          <t>ch15: 508-516, 518 (cranial dura splits into periorbita + dural sheath at optic foramen; subdural space potential/artefact 510; dura 0.35-0.5 mm, circular internal + longitudinal/oblique peripheral fibres, collagen 600-700 um as printed, 2-5 outer lamellae 510-511; arachnoid ~10 um, meningothelial multilaminar + trabeculae + corpora amylacea, ends at lamina cribrosa 512; pia-glia / glial mantle of Fuchs + septa + vessels between longitudinal and circular fibres 513; SAS scleral cul-de-sac behind lamina cribrosa, widest anteriorly, wider nasally 515) [scans 13.pdf] | v1.1.0 pages: 525-527 + 530-560.pdf/586.pdf; ch1: 26 (sellar-region dura: diaphragma sellae roof of hypophysis; cavernous sinus dural walls flanking sphenoid body, interconnected across tuberculum/dorsum sellae) | v1.3.0 sources: StatPearls NBK507907 (CN II, 2022) read in full</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -3793,7 +3793,7 @@
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)] | v1.1.0 enrichment 2026-10-24: from batch-3 pages: CRA-sheath relationships appended to blood_supply (CRA pierces dura 5-15.5 mm behind globe inferomedially; intravaginal course 0.9-2.5 mm mainly within the subarachnoid space; vertical nerve entry with right-angled bend; intravaginal pial branches near the arterial entry; intraorbital branches supply pia from globe to canal in half the nerves) + CRV intravaginal course longer than the artery (3.8-8 mm) with greater dural residence appended to venous_drainage (pp.525-527); bilingual keywords extended; validate 27/27 + pytest 10+14 green</t>
+          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)] | v1.1.0 enrichment 2026-10-24: from batch-3 pages: CRA-sheath relationships appended to blood_supply (CRA pierces dura 5-15.5 mm behind globe inferomedially; intravaginal course 0.9-2.5 mm mainly within the subarachnoid space; vertical nerve entry with right-angled bend; intravaginal pial branches near the arterial entry; intraorbital branches supply pia from globe to canal in half the nerves) + CRV intravaginal course longer than the artery (3.8-8 mm) with greater dural residence appended to venous_drainage (pp.525-527); bilingual keywords extended; validate 27/27 + pytest 10+14 green | v1.2.0 (2026-10-26) batch-4: sellar-region dural landmarks (diaphragma sellae + cavernous sinus walls) appended to location from owner-supplied printed 26; keywords +6; validate 27/27 green | v1.3.0 (2026-10-26) StatPearls round: ICP-propagation mechanism appended to clinical_importance (three meningeal sheaths continuous with brain -&gt; raised intracranial pressure propagates from intracranial to perineural subarachnoid space -&gt; papilloedema on fundoscopy; 25/25 quote checks); keywords +4; validate 27/27 green.</t>
         </is>
       </c>
     </row>
@@ -3830,7 +3830,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>ch15: 499, 515-518, 521 (septa invade with vessels ~4th month; 6-9 primary septa into sectors + dichotomous secondary septa; interseptal spaces rounded in human vs polygonal in other mammals 517; septa = tubes around fascicles, fenestrated; trabecula central vessel with muscular/elastic layers; astrocyte feet + basal lamina + invaginations 120-150 um (Anderson &amp; Hoyt 1969); astrocytes abut capillaries directly in chiasma 521; triangular glial septum separates ventromedial (crossing) from dorsolateral, marks start of decussation 518; support deficiency superior/inferior -&gt; early glaucomatous bowing (Quigley) 499) [scans 13.pdf] | v1.1.0 pages: 525, 529 + 530-560.pdf/586.pdf</t>
+          <t>ch15: 499, 515-518, 521 (septa invade with vessels ~4th month; 6-9 primary septa into sectors + dichotomous secondary septa; interseptal spaces rounded in human vs polygonal in other mammals 517; septa = tubes around fascicles, fenestrated; trabecula central vessel with muscular/elastic layers; astrocyte feet + basal lamina + invaginations 120-150 um (Anderson &amp; Hoyt 1969); astrocytes abut capillaries directly in chiasma 521; triangular glial septum separates ventromedial (crossing) from dorsolateral, marks start of decussation 518; support deficiency superior/inferior -&gt; early glaucomatous bowing (Quigley) 499) [scans 13.pdf] | v1.1.0 pages: 525, 529 + 530-560.pdf/586.pdf | v1.2.0 pages: ch15: 494 (Anderson 1969: laminar/postlaminar astrocyte layer thinner than prelaminar; oligodendrocyte columns in myelinated fascicles; lamina-cribrosa connective tissue continuous posteriorly with pial septae)</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -3900,7 +3900,7 @@
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)] | v1.1.0 enrichment 2026-10-24: from batch-3 pages: pial plexus centripetal branches each within a glial-coated connective-tissue core (p.525) + CRA intraneural branches anastomosing with the septal arteriolar/capillary system (p.529) + full intraseptal microvasculature account (large precapillaries/capillaries confined to septae in transverse and longitudinal polygonal units; extensive anastomosis, size non-uniformity, numbers increasing near posterior laminal bowing; anterior anastomosis with laminar vessels, posterior with intraorbital septal system — Lieberman/Maumenee/Green 1976) appended to blood_supply; bilingual keywords extended; validate 27/27 + pytest 10+14 green</t>
+          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)] | v1.1.0 enrichment 2026-10-24: from batch-3 pages: pial plexus centripetal branches each within a glial-coated connective-tissue core (p.525) + CRA intraneural branches anastomosing with the septal arteriolar/capillary system (p.529) + full intraseptal microvasculature account (large precapillaries/capillaries confined to septae in transverse and longitudinal polygonal units; extensive anastomosis, size non-uniformity, numbers increasing near posterior laminal bowing; anterior anastomosis with laminar vessels, posterior with intraorbital septal system — Lieberman/Maumenee/Green 1976) appended to blood_supply; bilingual keywords extended; validate 27/27 + pytest 10+14 green | v1.2.0 (2026-10-26) batch-5: owner text printed 494 (Fig 15.8) - laminar/postlaminar septal architecture appended to histology_summary: astrocytes separating fascicles thinner than prelaminar, myelinated fascicles contain oligodendrocyte columns, connective tissue of lamina cribrosa continuous posteriorly with pial septae; keywords +5; validate 27/27 + pytest green.</t>
         </is>
       </c>
     </row>
@@ -3937,7 +3937,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>ch15: 521-524, 527-534 (pial network double system + septal distribution exact = vessels 521; perichiasmal artery largest intracranial supply, origin superior hypophyseal (Hayreh 1963/Steele &amp; Blunt 1956) vs Dawson 1958 ophthalmic 522; intracanalicular OA sole supply, poor pial network vulnerable to shearing in skull fracture 524; intraorbital: CRA enters 5-15.5 mm behind globe, proximal centripetal vs distal axial, 3 sources, direct branches reach pia in 75% when OA crosses above (82-85% of cases) 524; venous drainage: pial veins + central retinal vein(s) (embryonic 2 channels beside hyaloid artery 3rd month; exit same aspect in 42%, vein anterior to artery in 81% (Fry 1930); intravaginal course 3.8-8 mm) + posterior central vein 527; cavernous sinus blockage does not block CRV flow 528; laminar circle of Zinn (1755)/Haller (1754) branches 1-4 + interfacial precapillaries vulnerable to raised IOP -&gt; disc haemorrhages (Ruskell 1984) 531; prelaminar scleral SPCA vs recurrent choroidal (only 10% choroidal origin, Lieberman 1976) + microvascular cuff 534; SNFL 5 supplies with CRA major 534; BBB incomplete at ONH (pars choroidalis) 534) [scans 13.pdf+14.pdf] | v1.1.0 pages: 525-526, 530, 533, 541, 543 + 530-560.pdf/586.pdf</t>
+          <t>ch15: 521-524, 527-534 (pial network double system + septal distribution exact = vessels 521; perichiasmal artery largest intracranial supply, origin superior hypophyseal (Hayreh 1963/Steele &amp; Blunt 1956) vs Dawson 1958 ophthalmic 522; intracanalicular OA sole supply, poor pial network vulnerable to shearing in skull fracture 524; intraorbital: CRA enters 5-15.5 mm behind globe, proximal centripetal vs distal axial, 3 sources, direct branches reach pia in 75% when OA crosses above (82-85% of cases) 524; venous drainage: pial veins + central retinal vein(s) (embryonic 2 channels beside hyaloid artery 3rd month; exit same aspect in 42%, vein anterior to artery in 81% (Fry 1930); intravaginal course 3.8-8 mm) + posterior central vein 527; cavernous sinus blockage does not block CRV flow 528; laminar circle of Zinn (1755)/Haller (1754) branches 1-4 + interfacial precapillaries vulnerable to raised IOP -&gt; disc haemorrhages (Ruskell 1984) 531; prelaminar scleral SPCA vs recurrent choroidal (only 10% choroidal origin, Lieberman 1976) + microvascular cuff 534; SNFL 5 supplies with CRA major 534; BBB incomplete at ONH (pars choroidalis) 534) [scans 13.pdf+14.pdf] | v1.1.0 pages: 525-526, 530, 533, 541, 543 + 530-560.pdf/586.pdf | v1.2.0 pages: ch11: 386 (Fig 11.13 Olver 1990 cast: temporal+medial SPCA bundles supply choroid AND retrolaminar nerve; paraoptic branches -&gt; circle of Zinn-Haller -&gt; pial branches to retrolaminar nerve + recurrent choroidal to peripapillary and peripheral vertical meridional choroid; triangular/trapezoid SPCA territories) | v1.3.0 sources: StatPearls NBK507907 + NBK542287 read in full</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -4007,7 +4007,7 @@
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)] | v1.1.0 enrichment 2026-10-24: batch-3 pages mined heavily: intraorbital layers block extended with the long-awaited p.525 material (pial plexus tortuous anastomoses reinforced at nerve-globe junction by scleral SPCA/circle of Zinn; centripetal branches within glial-coated cores; CRA origin variants relative to ophthalmic artery crossing; CRA course - dura piercing 5-15.5 mm inferomedially, intravaginal 0.9-2.5 mm in subarachnoid space, vertical entry + right-angled bend, ~5/3/8 intraorbital/intravaginal/intraneural branches; Hayreh 1963 stats - branches in all but 3.1%, none to lamina cribrosa, lacking intraorbital 47.8%/intravaginal 5.3%/intraneural 25%; collaterals superior/inferior per OA crossing, lateral rare vs Hughes 1954; CRA pial territory always inferior, superior least) + blood_supply extended with CRA wall structure (intima duplicated BM thickening with age; IEL irregular, disappears at lamina, absent from retinal arteries; media ~6 layers; adventitia continuous with septa) + GCA rule (only IEL-bearing vessels affected; retinal arteries spared - Cogan 1974) + Zinn-Haller frequency/form/position (pp.530-533) + chiasmal arterial supply (rich collateral anastomosis; Wollschlaeger 1971 630 specimens dorsal A1/ventral ICA-ACOMM with A2 contribution always per Perlmutter &amp; Rhoton 1976, no PCOMM/PCA/basilar contributions, superior hypophyseal + MCA feeders, dorsal/ventral classification) (pp.541-543) + GCA fact added to clinical; bilingual keywords extended; validate 27/27 + pytest 10+14 green</t>
+          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)] | v1.1.0 enrichment 2026-10-24: batch-3 pages mined heavily: intraorbital layers block extended with the long-awaited p.525 material (pial plexus tortuous anastomoses reinforced at nerve-globe junction by scleral SPCA/circle of Zinn; centripetal branches within glial-coated cores; CRA origin variants relative to ophthalmic artery crossing; CRA course - dura piercing 5-15.5 mm inferomedially, intravaginal 0.9-2.5 mm in subarachnoid space, vertical entry + right-angled bend, ~5/3/8 intraorbital/intravaginal/intraneural branches; Hayreh 1963 stats - branches in all but 3.1%, none to lamina cribrosa, lacking intraorbital 47.8%/intravaginal 5.3%/intraneural 25%; collaterals superior/inferior per OA crossing, lateral rare vs Hughes 1954; CRA pial territory always inferior, superior least) + blood_supply extended with CRA wall structure (intima duplicated BM thickening with age; IEL irregular, disappears at lamina, absent from retinal arteries; media ~6 layers; adventitia continuous with septa) + GCA rule (only IEL-bearing vessels affected; retinal arteries spared - Cogan 1974) + Zinn-Haller frequency/form/position (pp.530-533) + chiasmal arterial supply (rich collateral anastomosis; Wollschlaeger 1971 630 specimens dorsal A1/ventral ICA-ACOMM with A2 contribution always per Perlmutter &amp; Rhoton 1976, no PCOMM/PCA/basilar contributions, superior hypophyseal + MCA feeders, dorsal/ventral classification) (pp.541-543) + GCA fact added to clinical; bilingual keywords extended; validate 27/27 + pytest 10+14 green | v1.2.0 (2026-10-26) batch-5: owner text printed 386 (ch.11 Fig 11.13) - Olver/Spalton/McCartney 1990 posterior-pole vascular cast appended to blood_supply: SPCA dual supply (choroid + retrolaminar nerve), Zinn-Haller outflow to pial and recurrent choroidal branches incl. peripheral vertical meridional choroid, triangular/trapezoid choroidal territories; keywords +7; pages screened not cited: 30 (eyelids), 192 (trigeminal ganglion, ON in Fig 5.16 label only), 283 (Schlemm/sulcus), 361 (ciliary ageing), 403 (ciliary vessels), 665-693 bibliography (no anatomical facts; relevant ON literature already cited in-text); validate 27/27 + pytest green. | batch-6 screening (2026-10-26): owner text printed 390 (Fig 11.13 contd q-t - choroidal venous casts: collecting venules, vortex tributaries, venulo-venular anastomoses), 396 (choriocapillaris ultrastructure - 60-80nm fenestrations, pericytes, leaky discontinuous zonulae occludentes, Bruch's membrane 5 layers), 666 + 675 (bibliography; confirms primary refs already cited in-card: Anderson 1969b 82:800, Anderson &amp; Braverman 1976, Anderson/Hoyt/Hogan 1967) - choroid-domain or bibliography content, no optic-nerve facts, not cited per scope rule; material flagged for a future Choroid category. Pages 718-719/722-723 NOT received (second message truncation) - outstanding. | v1.3.0 (2026-10-26) StatPearls round: teaching-source corroboration appended to blood_supply (ophthalmic artery = first branch of ICA arising just distal to cavernous sinus; within the optic canal it courses inferior and lateral to the nerve before its intraorbital crossing; circle of Willis encircles the opto-chiasmatic region with branches perfusing intracranial nerve and chiasm; 25/25 quote checks); keywords +4; validate 27/27 green. Cards ON-002/ON-004 unchanged - corroborating StatPearls facts already covered by Wolff citations.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Enrich lens+vitreous to v1.1.0; add 2 optic references; fix component registry
</commit_message>
<xml_diff>
--- a/Anatomy_Extraction_Master_Tracker_v2.xlsx
+++ b/Anatomy_Extraction_Master_Tracker_v2.xlsx
@@ -1052,7 +1052,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U28"/>
+  <dimension ref="A1:U40"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="5"/>
   <sheetData>
     <row r="1">
@@ -3509,7 +3509,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>ch15: 495-499, 508-509, 515-521, 524 (papillomotor/centrifugal fibres + 800-1200 fascicles (Deyl 1895) + axon estimates Polyak/Oppel/Kupfer 515; axon diameters 0.7-10 um, 92% &lt;1 um, microtubules 20-25 nm (Anderson &amp; Hoyt 1969) 521/515; retrolaminar myelination doubles diameter 1.5-&gt;3.0 mm (Minckler 1976) 499; orbit relations incl. ciliary ganglion + CRA entry ~12 mm behind eye 508; scleral canal 0.5 mm 505; orbital length 3 cm 524) [scans 13.pdf+14.pdf] | v1.1.0 pages: 540-541 + 530-560.pdf/586.pdf; ch1: 23, 24, 25, 26 (bony optic canal between two roots of lesser wing; chiasmal sulcus rarely contacting chiasm; jugum sphenoidale; anterior/middle clinoid + caroticoclinoid foramen; cavernous sinus extent &amp; intercavernous connections; diaphragma sellae; SOF vs optic canal); ch5: 190 (cavernous lateral wall: III/IV/V1/V2, VI free inferolateral to ICA) | v1.3.0 sources: StatPearls NBK507907 (CN II, 2022) + NBK542287 (Optic Chiasm, 2023) read in full</t>
+          <t>ch15: 495-499, 508-509, 515-521, 524 (papillomotor/centrifugal fibres + 800-1200 fascicles (Deyl 1895) + axon estimates Polyak/Oppel/Kupfer 515; axon diameters 0.7-10 um, 92% &lt;1 um, microtubules 20-25 nm (Anderson &amp; Hoyt 1969) 521/515; retrolaminar myelination doubles diameter 1.5-&gt;3.0 mm (Minckler 1976) 499; orbit relations incl. ciliary ganglion + CRA entry ~12 mm behind eye 508; scleral canal 0.5 mm 505; orbital length 3 cm 524) [scans 13.pdf+14.pdf] | v1.1.0 pages: 540-541 + 530-560.pdf/586.pdf</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -3579,7 +3579,7 @@
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)] | v1.1.0 enrichment 2026-10-24: batch-3 pages (printed 525, 535-545, 586-590 from scans 530-560.pdf = printed 525-550 verified 1:1 + 586.pdf = printed 586-590 verified 1:1) read visually and mined; fibre topography of the proximal nerve appended to histology (crossed/uncrossed separation begins proximally with crossing fibres medial to the pial septum end; nasal fibres form a quadrilateral sheet; inferior nasal fibres loop forward into the contralateral proximal nerve up to 3 mm = knee of Wilbrand) + clinical consequence (proximal nerve compression affects both eyes' fields; pituitary chiasmal involvement heralded by upper bitemporal quadrantanopia, pp.540-541); bilingual keywords extended; validate 27/27 + pytest 10+14 green | v1.2.0 (2026-10-26) batch-4: skull-base relations &amp; cavernous sinus topography from owner-supplied text (printed 23-26, 190) - bony canal (two roots of lesser wing, direction forwards/laterally/downwards), chiasmal sulcus above/behind -&gt; chiasm elevation by sellar expansion, anterior clinoid + caroticoclinoid foramen, cavernous sinus extent pp.23-26; localization contrast: CN II outside sinus whose lateral wall carries III/IV/V1/V2 with VI free (p.190) -&gt; vision spared in cavernous lesions; pages 22, 27-29, 189, 191, 282, 359-360 screened: no optic-nerve facts, not cited; bilingual keywords +20; validate 27/27 + pytest 10+14 green | v1.3.0 (2026-10-26) StatPearls round: both articles fetched via /sites/books/ and read in FULL (2,597 + 5,014 words) with 25/25 literal quote checks passed before writing. definition: explicit synaptic targets (SCN circadian, LGN, pretectal, superior colliculus) + afferent limb of light and accommodation reflexes; location: chiasm ~10 mm above pituitary in suprasellar cistern, adjacent to third-ventricle anterior wall/floor junction; clinical: chiasm position variants (normo-fixed 85% / pre-fixed 7.5% / post-fixed 8%, cadaver study) + lesion localisation (pre-chiasmal ipsilateral monocular; pituitary macroadenoma compresses inferior chiasm -&gt; superior temporal loss before bitemporal; optic pathway glioma 3-5% paediatric / 6.6-20% NF1) + RAPD/Marcus Gunn with swinging flashlight test; histology: unmyelinated-until-lamina rationale (retinal light path), optic stalk 4th week -&gt; nerve, hyaloid vessels -&gt; CRA/CRV, myelination timeline (LGN 5mo -&gt; tract 6mo -&gt; chiasm 6-7mo -&gt; nerve 8mo; crossed 7-8wk, uncrossed ~11wk) + modern-imaging caveat on knees of Wilbrand (failed identification, shifting rejection in normals, possible sequela of long-term monocular neuropathy). Registry +2 statpearls entries (14 total). validate 27/27 + pytest green.</t>
+          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)] | v1.1.0 enrichment 2026-10-24: batch-3 pages (printed 525, 535-545, 586-590 from scans 530-560.pdf = printed 525-550 verified 1:1 + 586.pdf = printed 586-590 verified 1:1) read visually and mined; fibre topography of the proximal nerve appended to histology (crossed/uncrossed separation begins proximally with crossing fibres medial to the pial septum end; nasal fibres form a quadrilateral sheet; inferior nasal fibres loop forward into the contralateral proximal nerve up to 3 mm = knee of Wilbrand) + clinical consequence (proximal nerve compression affects both eyes' fields; pituitary chiasmal involvement heralded by upper bitemporal quadrantanopia, pp.540-541); bilingual keywords extended; validate 27/27 + pytest 10+14 green</t>
         </is>
       </c>
     </row>
@@ -3616,7 +3616,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>ch15: 503-508, 528-534 (disc area 0.86-5.54 mm2 mean 2.69±0.7 + macrodiscs &gt;4.09/microdiscs &lt;1.29 (Jonas/Gusek/Naumann 1988, 1991) + Table 15.1 full metrics 505; lamina area 2.88±0.84 mm2 + pore count 227±36 (Jonas 1991) + cup metrics + rim broadest inferior-&gt;superior-&gt;nasal-&gt;temporal, narrowest temporal horizontal in 99.2% 506; cup/disc ratio median 0.3, vertical lower in 93.2%, asymmetry &gt;0.2 diagnostic; parapapillary zones alpha 84.4%/beta 15.2% + POAG alpha 0.65/beta 0.79 507; RNFL visibility order + axon loss 4-5000/yr 508; ONH watershed + zonal arterial supply + venous drainage + opticociliary veins 528-534) [scans 13.pdf+14.pdf] | v1.1.0 pages: 530, 533, 534-535 + 530-560.pdf/586.pdf | v1.2.0 pages: ch15: 494-495 (Anderson 1969 Fig 15.8: prelaminar astrocytic tubes with perpendicular astrocytes + intratubular capillaries; laminar fascicle astrocyte layer + connective-tissue mantle; postlaminar oligodendrocyte columns; border tissue of Jacoby cuff -&gt; intermediary tissue of Kuhnt forwards, glial mantle backwards)</t>
+          <t>ch15: 503-508, 528-534 (disc area 0.86-5.54 mm2 mean 2.69±0.7 + macrodiscs &gt;4.09/microdiscs &lt;1.29 (Jonas/Gusek/Naumann 1988, 1991) + Table 15.1 full metrics 505; lamina area 2.88±0.84 mm2 + pore count 227±36 (Jonas 1991) + cup metrics + rim broadest inferior-&gt;superior-&gt;nasal-&gt;temporal, narrowest temporal horizontal in 99.2% 506; cup/disc ratio median 0.3, vertical lower in 93.2%, asymmetry &gt;0.2 diagnostic; parapapillary zones alpha 84.4%/beta 15.2% + POAG alpha 0.65/beta 0.79 507; RNFL visibility order + axon loss 4-5000/yr 508; ONH watershed + zonal arterial supply + venous drainage + opticociliary veins 528-534) [scans 13.pdf+14.pdf] | v1.1.0 pages: 530, 533, 534-535 + 530-560.pdf/586.pdf</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -3686,7 +3686,7 @@
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)] | v1.1.0 enrichment 2026-10-24: from batch-3 pages (525, 535-545, 586-590): circle of Zinn-Haller frequency dispute (Olver 1990 frequently present vs Hayreh small proportion; often incomplete Levitzky &amp; Henkind 1969; ABSENT in sub-human primates Hayreh 1964; horizontal-ellipse intrascleral anastomosis of medial+lateral paraoptic SPCA branches; paraoptic replacements when absent) + positional variants (apposed/distant/anterior intrascleral/posterior extrascleral; axial position on SEM) appended to blood_supply; marginal tissue of Kuhnt glial 'gasket' tight junctions appended to histology (Tso/Shih/McLean 1975); incomplete ONH blood-brain barrier with HRP tracer route choroid-&gt;prelaminar-&gt;lamina septa-&gt;retrolaminar + implications for optic pits and papilloedema appended to clinical (pp.534-535); bilingual keywords extended; validate 27/27 + pytest 10+14 green | v1.2.0 (2026-10-26) batch-5: owner text printed 494 (+495 continuation verified visually from scan render) - prelaminar astrocytic-tube architecture (bundles + perpendicular astrocytes, capillaries within tubes), peripheral astrocyte cuff = border tissue of Jacoby continuing forwards as intermediary tissue of Kuhnt and backwards in continuity with glial mantle deep to pia, laminar astrocyte layer + mantle of connective tissue (collagen/elastic/fibroblasts/capillaries) thinner than prelaminar, postlaminar myelination with columns of oligodendrocytes + few astrocytes, glial separation rule (Anderson/Hoyt/Hogan 1967) with CRA-adventitia exception (Ikui 1964) appended to layers[1..3]; keywords +10; validate 27/27 + pytest green.</t>
+          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)] | v1.1.0 enrichment 2026-10-24: from batch-3 pages (525, 535-545, 586-590): circle of Zinn-Haller frequency dispute (Olver 1990 frequently present vs Hayreh small proportion; often incomplete Levitzky &amp; Henkind 1969; ABSENT in sub-human primates Hayreh 1964; horizontal-ellipse intrascleral anastomosis of medial+lateral paraoptic SPCA branches; paraoptic replacements when absent) + positional variants (apposed/distant/anterior intrascleral/posterior extrascleral; axial position on SEM) appended to blood_supply; marginal tissue of Kuhnt glial 'gasket' tight junctions appended to histology (Tso/Shih/McLean 1975); incomplete ONH blood-brain barrier with HRP tracer route choroid-&gt;prelaminar-&gt;lamina septa-&gt;retrolaminar + implications for optic pits and papilloedema appended to clinical (pp.534-535); bilingual keywords extended; validate 27/27 + pytest 10+14 green</t>
         </is>
       </c>
     </row>
@@ -3723,7 +3723,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>ch15: 508-516, 518 (cranial dura splits into periorbita + dural sheath at optic foramen; subdural space potential/artefact 510; dura 0.35-0.5 mm, circular internal + longitudinal/oblique peripheral fibres, collagen 600-700 um as printed, 2-5 outer lamellae 510-511; arachnoid ~10 um, meningothelial multilaminar + trabeculae + corpora amylacea, ends at lamina cribrosa 512; pia-glia / glial mantle of Fuchs + septa + vessels between longitudinal and circular fibres 513; SAS scleral cul-de-sac behind lamina cribrosa, widest anteriorly, wider nasally 515) [scans 13.pdf] | v1.1.0 pages: 525-527 + 530-560.pdf/586.pdf; ch1: 26 (sellar-region dura: diaphragma sellae roof of hypophysis; cavernous sinus dural walls flanking sphenoid body, interconnected across tuberculum/dorsum sellae) | v1.3.0 sources: StatPearls NBK507907 (CN II, 2022) read in full</t>
+          <t>ch15: 508-516, 518 (cranial dura splits into periorbita + dural sheath at optic foramen; subdural space potential/artefact 510; dura 0.35-0.5 mm, circular internal + longitudinal/oblique peripheral fibres, collagen 600-700 um as printed, 2-5 outer lamellae 510-511; arachnoid ~10 um, meningothelial multilaminar + trabeculae + corpora amylacea, ends at lamina cribrosa 512; pia-glia / glial mantle of Fuchs + septa + vessels between longitudinal and circular fibres 513; SAS scleral cul-de-sac behind lamina cribrosa, widest anteriorly, wider nasally 515) [scans 13.pdf] | v1.1.0 pages: 525-527 + 530-560.pdf/586.pdf</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -3793,7 +3793,7 @@
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)] | v1.1.0 enrichment 2026-10-24: from batch-3 pages: CRA-sheath relationships appended to blood_supply (CRA pierces dura 5-15.5 mm behind globe inferomedially; intravaginal course 0.9-2.5 mm mainly within the subarachnoid space; vertical nerve entry with right-angled bend; intravaginal pial branches near the arterial entry; intraorbital branches supply pia from globe to canal in half the nerves) + CRV intravaginal course longer than the artery (3.8-8 mm) with greater dural residence appended to venous_drainage (pp.525-527); bilingual keywords extended; validate 27/27 + pytest 10+14 green | v1.2.0 (2026-10-26) batch-4: sellar-region dural landmarks (diaphragma sellae + cavernous sinus walls) appended to location from owner-supplied printed 26; keywords +6; validate 27/27 green | v1.3.0 (2026-10-26) StatPearls round: ICP-propagation mechanism appended to clinical_importance (three meningeal sheaths continuous with brain -&gt; raised intracranial pressure propagates from intracranial to perineural subarachnoid space -&gt; papilloedema on fundoscopy; 25/25 quote checks); keywords +4; validate 27/27 green.</t>
+          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)] | v1.1.0 enrichment 2026-10-24: from batch-3 pages: CRA-sheath relationships appended to blood_supply (CRA pierces dura 5-15.5 mm behind globe inferomedially; intravaginal course 0.9-2.5 mm mainly within the subarachnoid space; vertical nerve entry with right-angled bend; intravaginal pial branches near the arterial entry; intraorbital branches supply pia from globe to canal in half the nerves) + CRV intravaginal course longer than the artery (3.8-8 mm) with greater dural residence appended to venous_drainage (pp.525-527); bilingual keywords extended; validate 27/27 + pytest 10+14 green</t>
         </is>
       </c>
     </row>
@@ -3830,7 +3830,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>ch15: 499, 515-518, 521 (septa invade with vessels ~4th month; 6-9 primary septa into sectors + dichotomous secondary septa; interseptal spaces rounded in human vs polygonal in other mammals 517; septa = tubes around fascicles, fenestrated; trabecula central vessel with muscular/elastic layers; astrocyte feet + basal lamina + invaginations 120-150 um (Anderson &amp; Hoyt 1969); astrocytes abut capillaries directly in chiasma 521; triangular glial septum separates ventromedial (crossing) from dorsolateral, marks start of decussation 518; support deficiency superior/inferior -&gt; early glaucomatous bowing (Quigley) 499) [scans 13.pdf] | v1.1.0 pages: 525, 529 + 530-560.pdf/586.pdf | v1.2.0 pages: ch15: 494 (Anderson 1969: laminar/postlaminar astrocyte layer thinner than prelaminar; oligodendrocyte columns in myelinated fascicles; lamina-cribrosa connective tissue continuous posteriorly with pial septae)</t>
+          <t>ch15: 499, 515-518, 521 (septa invade with vessels ~4th month; 6-9 primary septa into sectors + dichotomous secondary septa; interseptal spaces rounded in human vs polygonal in other mammals 517; septa = tubes around fascicles, fenestrated; trabecula central vessel with muscular/elastic layers; astrocyte feet + basal lamina + invaginations 120-150 um (Anderson &amp; Hoyt 1969); astrocytes abut capillaries directly in chiasma 521; triangular glial septum separates ventromedial (crossing) from dorsolateral, marks start of decussation 518; support deficiency superior/inferior -&gt; early glaucomatous bowing (Quigley) 499) [scans 13.pdf] | v1.1.0 pages: 525, 529 + 530-560.pdf/586.pdf</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -3900,7 +3900,7 @@
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)] | v1.1.0 enrichment 2026-10-24: from batch-3 pages: pial plexus centripetal branches each within a glial-coated connective-tissue core (p.525) + CRA intraneural branches anastomosing with the septal arteriolar/capillary system (p.529) + full intraseptal microvasculature account (large precapillaries/capillaries confined to septae in transverse and longitudinal polygonal units; extensive anastomosis, size non-uniformity, numbers increasing near posterior laminal bowing; anterior anastomosis with laminar vessels, posterior with intraorbital septal system — Lieberman/Maumenee/Green 1976) appended to blood_supply; bilingual keywords extended; validate 27/27 + pytest 10+14 green | v1.2.0 (2026-10-26) batch-5: owner text printed 494 (Fig 15.8) - laminar/postlaminar septal architecture appended to histology_summary: astrocytes separating fascicles thinner than prelaminar, myelinated fascicles contain oligodendrocyte columns, connective tissue of lamina cribrosa continuous posteriorly with pial septae; keywords +5; validate 27/27 + pytest green.</t>
+          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)] | v1.1.0 enrichment 2026-10-24: from batch-3 pages: pial plexus centripetal branches each within a glial-coated connective-tissue core (p.525) + CRA intraneural branches anastomosing with the septal arteriolar/capillary system (p.529) + full intraseptal microvasculature account (large precapillaries/capillaries confined to septae in transverse and longitudinal polygonal units; extensive anastomosis, size non-uniformity, numbers increasing near posterior laminal bowing; anterior anastomosis with laminar vessels, posterior with intraorbital septal system — Lieberman/Maumenee/Green 1976) appended to blood_supply; bilingual keywords extended; validate 27/27 + pytest 10+14 green</t>
         </is>
       </c>
     </row>
@@ -3937,7 +3937,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>ch15: 521-524, 527-534 (pial network double system + septal distribution exact = vessels 521; perichiasmal artery largest intracranial supply, origin superior hypophyseal (Hayreh 1963/Steele &amp; Blunt 1956) vs Dawson 1958 ophthalmic 522; intracanalicular OA sole supply, poor pial network vulnerable to shearing in skull fracture 524; intraorbital: CRA enters 5-15.5 mm behind globe, proximal centripetal vs distal axial, 3 sources, direct branches reach pia in 75% when OA crosses above (82-85% of cases) 524; venous drainage: pial veins + central retinal vein(s) (embryonic 2 channels beside hyaloid artery 3rd month; exit same aspect in 42%, vein anterior to artery in 81% (Fry 1930); intravaginal course 3.8-8 mm) + posterior central vein 527; cavernous sinus blockage does not block CRV flow 528; laminar circle of Zinn (1755)/Haller (1754) branches 1-4 + interfacial precapillaries vulnerable to raised IOP -&gt; disc haemorrhages (Ruskell 1984) 531; prelaminar scleral SPCA vs recurrent choroidal (only 10% choroidal origin, Lieberman 1976) + microvascular cuff 534; SNFL 5 supplies with CRA major 534; BBB incomplete at ONH (pars choroidalis) 534) [scans 13.pdf+14.pdf] | v1.1.0 pages: 525-526, 530, 533, 541, 543 + 530-560.pdf/586.pdf | v1.2.0 pages: ch11: 386 (Fig 11.13 Olver 1990 cast: temporal+medial SPCA bundles supply choroid AND retrolaminar nerve; paraoptic branches -&gt; circle of Zinn-Haller -&gt; pial branches to retrolaminar nerve + recurrent choroidal to peripapillary and peripheral vertical meridional choroid; triangular/trapezoid SPCA territories) | v1.3.0 sources: StatPearls NBK507907 + NBK542287 read in full</t>
+          <t>ch15: 521-524, 527-534 (pial network double system + septal distribution exact = vessels 521; perichiasmal artery largest intracranial supply, origin superior hypophyseal (Hayreh 1963/Steele &amp; Blunt 1956) vs Dawson 1958 ophthalmic 522; intracanalicular OA sole supply, poor pial network vulnerable to shearing in skull fracture 524; intraorbital: CRA enters 5-15.5 mm behind globe, proximal centripetal vs distal axial, 3 sources, direct branches reach pia in 75% when OA crosses above (82-85% of cases) 524; venous drainage: pial veins + central retinal vein(s) (embryonic 2 channels beside hyaloid artery 3rd month; exit same aspect in 42%, vein anterior to artery in 81% (Fry 1930); intravaginal course 3.8-8 mm) + posterior central vein 527; cavernous sinus blockage does not block CRV flow 528; laminar circle of Zinn (1755)/Haller (1754) branches 1-4 + interfacial precapillaries vulnerable to raised IOP -&gt; disc haemorrhages (Ruskell 1984) 531; prelaminar scleral SPCA vs recurrent choroidal (only 10% choroidal origin, Lieberman 1976) + microvascular cuff 534; SNFL 5 supplies with CRA major 534; BBB incomplete at ONH (pars choroidalis) 534) [scans 13.pdf+14.pdf] | v1.1.0 pages: 525-526, 530, 533, 541, 543 + 530-560.pdf/586.pdf</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -4007,7 +4007,1291 @@
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)] | v1.1.0 enrichment 2026-10-24: batch-3 pages mined heavily: intraorbital layers block extended with the long-awaited p.525 material (pial plexus tortuous anastomoses reinforced at nerve-globe junction by scleral SPCA/circle of Zinn; centripetal branches within glial-coated cores; CRA origin variants relative to ophthalmic artery crossing; CRA course - dura piercing 5-15.5 mm inferomedially, intravaginal 0.9-2.5 mm in subarachnoid space, vertical entry + right-angled bend, ~5/3/8 intraorbital/intravaginal/intraneural branches; Hayreh 1963 stats - branches in all but 3.1%, none to lamina cribrosa, lacking intraorbital 47.8%/intravaginal 5.3%/intraneural 25%; collaterals superior/inferior per OA crossing, lateral rare vs Hughes 1954; CRA pial territory always inferior, superior least) + blood_supply extended with CRA wall structure (intima duplicated BM thickening with age; IEL irregular, disappears at lamina, absent from retinal arteries; media ~6 layers; adventitia continuous with septa) + GCA rule (only IEL-bearing vessels affected; retinal arteries spared - Cogan 1974) + Zinn-Haller frequency/form/position (pp.530-533) + chiasmal arterial supply (rich collateral anastomosis; Wollschlaeger 1971 630 specimens dorsal A1/ventral ICA-ACOMM with A2 contribution always per Perlmutter &amp; Rhoton 1976, no PCOMM/PCA/basilar contributions, superior hypophyseal + MCA feeders, dorsal/ventral classification) (pp.541-543) + GCA fact added to clinical; bilingual keywords extended; validate 27/27 + pytest 10+14 green | v1.2.0 (2026-10-26) batch-5: owner text printed 386 (ch.11 Fig 11.13) - Olver/Spalton/McCartney 1990 posterior-pole vascular cast appended to blood_supply: SPCA dual supply (choroid + retrolaminar nerve), Zinn-Haller outflow to pial and recurrent choroidal branches incl. peripheral vertical meridional choroid, triangular/trapezoid choroidal territories; keywords +7; pages screened not cited: 30 (eyelids), 192 (trigeminal ganglion, ON in Fig 5.16 label only), 283 (Schlemm/sulcus), 361 (ciliary ageing), 403 (ciliary vessels), 665-693 bibliography (no anatomical facts; relevant ON literature already cited in-text); validate 27/27 + pytest green. | batch-6 screening (2026-10-26): owner text printed 390 (Fig 11.13 contd q-t - choroidal venous casts: collecting venules, vortex tributaries, venulo-venular anastomoses), 396 (choriocapillaris ultrastructure - 60-80nm fenestrations, pericytes, leaky discontinuous zonulae occludentes, Bruch's membrane 5 layers), 666 + 675 (bibliography; confirms primary refs already cited in-card: Anderson 1969b 82:800, Anderson &amp; Braverman 1976, Anderson/Hoyt/Hogan 1967) - choroid-domain or bibliography content, no optic-nerve facts, not cited per scope rule; material flagged for a future Choroid category. Pages 718-719/722-723 NOT received (second message truncation) - outstanding. | v1.3.0 (2026-10-26) StatPearls round: teaching-source corroboration appended to blood_supply (ophthalmic artery = first branch of ICA arising just distal to cavernous sinus; within the optic canal it courses inferior and lateral to the nerve before its intraorbital crossing; circle of Willis encircles the opto-chiasmatic region with branches perfusing intracranial nerve and chiasm; 25/25 quote checks); keywords +4; validate 27/27 green. Cards ON-002/ON-004 unchanged - corroborating StatPearls facts already covered by Wolff citations.</t>
+          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)] | v1.1.0 enrichment 2026-10-24: batch-3 pages mined heavily: intraorbital layers block extended with the long-awaited p.525 material (pial plexus tortuous anastomoses reinforced at nerve-globe junction by scleral SPCA/circle of Zinn; centripetal branches within glial-coated cores; CRA origin variants relative to ophthalmic artery crossing; CRA course - dura piercing 5-15.5 mm inferomedially, intravaginal 0.9-2.5 mm in subarachnoid space, vertical entry + right-angled bend, ~5/3/8 intraorbital/intravaginal/intraneural branches; Hayreh 1963 stats - branches in all but 3.1%, none to lamina cribrosa, lacking intraorbital 47.8%/intravaginal 5.3%/intraneural 25%; collaterals superior/inferior per OA crossing, lateral rare vs Hughes 1954; CRA pial territory always inferior, superior least) + blood_supply extended with CRA wall structure (intima duplicated BM thickening with age; IEL irregular, disappears at lamina, absent from retinal arteries; media ~6 layers; adventitia continuous with septa) + GCA rule (only IEL-bearing vessels affected; retinal arteries spared - Cogan 1974) + Zinn-Haller frequency/form/position (pp.530-533) + chiasmal arterial supply (rich collateral anastomosis; Wollschlaeger 1971 630 specimens dorsal A1/ventral ICA-ACOMM with A2 contribution always per Perlmutter &amp; Rhoton 1976, no PCOMM/PCA/basilar contributions, superior hypophyseal + MCA feeders, dorsal/ventral classification) (pp.541-543) + GCA fact added to clinical; bilingual keywords extended; validate 27/27 + pytest 10+14 green</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>LNS-001</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Lens</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Crystalline Lens (whole organ)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>ch12: 411-414, 432-434 | biometry: equatorial 9-10 mm adult / 6.5 mm birth; axial 3.5-4.0 birth -&gt; 4.75-5.0 extreme age; anterior radius 10 mm [8-14], posterior 6 mm [4.5-7.5]; RI 1.39 vs aqueous 1.33; ~15 D of ~40 D total; growth +29 um/yr sagittal, first 2 decades equatorial + nuclear compaction; avascular; glycolysis chief path, 3% aerobic (epithelium+superficial cortex) = up to 20% energy; aqueous glucose ~100 mg%, vitreous 90 mg%; Wieger ring 8-9 mm, Berger space, patellar fossa</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>lens.json</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff ch.12 scans 421-430/431-444/445-453.pdf)</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 39/39, 2026-10-26, incl. v1.1.0)</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>v1.1.0; created 2026-10-26 from Wolff Ch.12 12.1 (whole-lens blocks). Fields: definition/location/layers (capsule-epithelium-cortex-nucleus)/blood_supply/histology/clinical. Clinical: accommodation 15-16 D birth -&gt; half at 25 y -&gt; &lt;=2 D at 50 (presbyopia); cataract mechanism (irregularity, membrane degradation, crystallin aggregates, no nuclear protein turnover -&gt; brunescent nuclear cataract); contusion opacity recedes at ~2x growth speed -&gt; dating of trauma; zones of optical discontinuity for slit-lamp ageing/localisation; aphakia ~25 D loss | enrichment v1.1.0 APPLIED 2026-10-26: post-Wolff evidence merged into fields; refs: strenk_1999, jones_2005_grin, schachar_1992</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>LNS-002</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Lens</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Lens Capsule</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>ch12: 414-416, 439-441 | thickest basement membrane in body; thickness 15.5 um anterior pole / 2.8 um posterior pole (Fincham), increases anteriorly with age; up to ~40 lamellae x ~40 nm, collagen fibrils ~2.5 nm; type IV collagen (+ types I/III) in glycoprotein matrix (Kefalides/Dische), ~10% carbohydrate, PAS+; no elastin but elastic behaviour (superhelical collagen; Fisher &amp; Wakely, Fisher &amp; Hayes); zonular lamella of Berger 0.6-0.9 um, 1.0-1.7 um lateral to anterior zonular insertions; zonular fibrils into capsule 0.6-1.6 um deep (fibres ~2 um); permeability: water/ions free, molecules &lt; Hb 66.7 kDa diffuse (Fischer), blocks Hb/albumin 70 kDa + bacteria/inflammatory cells</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>lens-capsule.json</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff ch.12 scans 421-430/431-444/445-453.pdf)</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 39/39, 2026-10-26, incl. v1.1.0)</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>v1.1.0; created 2026-10-26 (capsule + zonular-lamella block of 12.1). Clinical: elastic recoil used in ECCE + Nd:YAG capsulotomy; posterior pole thinness -&gt; surgical delicacy; Fisher 1971 (capsular elasticity loss = major presbyopia factor) vs Weale 1982 question; zonule-free area 8 mm at 20 y -&gt; 6.5 mm 8th decade (or 5.5 mm) (Farnsworth &amp; Shine; Stark &amp; Streeten) -&gt; capsulotomy may meet zonular insertions; Wieger hyaloideocapsular ring 8-9 mm | enrichment v1.1.0 APPLIED 2026-10-26: post-Wolff evidence merged into fields; refs: schachar_1992, aao_bcsc_lens</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>LNS-003</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Lens</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Lens Epithelium</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>ch12: 416-423, 432-434 | ~500,000 cells; central density 5,009/mm2 men vs 5,781/mm2 women, declines with age; 3 zones: central (large flat, scattered mitoses), pre-equatorial germinative (small, compact, highest DNA synthesis + mitoses, circadian rhythm, light-enhanced, UV-shielded behind iris), equatorial bow (180-deg rotation into fibres); organelle-rich (mito, RER, ribosomes, Golgi, glycogen); desmosomes + gap junctions laterally, hemidesmosomes basally into capsule, apical junctional complexes to fibre apices; alpha-crystallin only (beta/gamma at fibre differentiation); pump-leak Na+/K+-ATPase seat</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>lens-epithelium.json</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff ch.12 scans 421-430/431-444/445-453.pdf)</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 39/39, 2026-10-26, incl. v1.1.0)</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>v1.1.0; created 2026-10-26 (epithelium block of 12.1 + pump-leak block). Clinical: residual LECs -&gt; PCO, Elschnig pearls, Soemmering ring -&gt; capsular polishing + Nd:YAG capsulotomy rationale; germinative zone target of radiation/UV -&gt; anterior subcapsular cataract; iris shielding relevance in aniridia/coloboma/chronic dilatation; epithelial pump failure -&gt; osmotic fibre swelling + cataract | enrichment v1.1.0 APPLIED 2026-10-26: post-Wolff evidence merged into fields; refs: aao_bcsc_lens</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>LNS-004</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Lens</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Lens Fibres</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>ch12: 421-432 | strap-like/spindle hexagonal cells; width 10-12 um, thickness 1.5-2 um at adult equator; primary fibres &lt;250 um, adult &gt;7 mm; highest protein of any cell ~35% wet weight; alpha + beta + gamma crystallins; nuclear bow S/C curve (Fig 12.21), anucleation ~150 um into cortex, nucleated zone 300-500 um (Kuwabara 1975); cortex/nucleus division = fetal/postnatal junction (6.5 mm at birth); thinner posteriorly -&gt; anterior cortex thicker (Kuszak 1984,1989); growth by rows not width in primates; fibre fusions pentagonal -&gt; positional info (Kuszak 1989); tips flare+curve at sutures (no taper in primates), overlap ~70 um, flattening 2 um cortex / 5 um nucleus; membrane specializations by depth: superficial 8-10 layers ball-and-socket on short sides; mid-cortex maximal ball-and-socket (resists zonular stress), layer-internal firm + layer-external loose -&gt; accommodation sliding; deep cortex miniature ball-and-socket on broad faces; nucleus tongue-and-groove + furrowed membrane domains 2-9 um2 with microvilli 0.14 um x 1.25-4.75 um; new fibres smooth -&gt; microplicae (Fig 12.32); gap junctions &lt;2 nm gap, 16-18 nm pentalaminar; human 5% of lateral membrane (frog 15%, rat 30%, chick 60%), absent at tips/sutural zone, density rises toward equator; MP70 gap junctions cortex, MP26 square arrays nucleus (Zampighi 1989); square arrays 11-13 nm asymmetrical; fusions throughout cortex+nucleus (Figs 12.22, 12.30-12.35)</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>lens-fibres.json</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff ch.12 scans 431-444.pdf)</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 39/39, 2026-10-26, incl. v1.1.0)</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>v1.1.0; created 2026-10-26 (fibres + membrane-specializations + junctions blocks of 12.1). Clinical: transparency = packing regularity + extracellular space &lt;1% volume; interlocking allows fibre sliding/flexing -&gt; accommodation requirement; suture planes = increased spherical aberration (Kuszak, Sivak &amp; Weeheim 1991); growth shells -&gt; zones of optical discontinuity (Kuszak, Brown &amp; Deutsch 1993); gap junctions = metabolic lifeline of organelle-free fibres, no crystalline&lt;-&gt;low-resistance transformation (Goodenough 1979); square arrays -&gt; extracellular drainage to sutures, transcytosis anteriorly/diffusion posteriorly (Kuszak 1993); contusion opacity recedes at ~2x growth speed (Brown 1988) | enrichment v1.1.0 APPLIED 2026-10-26: post-Wolff evidence merged into fields; refs: li_2022_aqp0_adhesion (AQP0 adhesion + connexin identities), cheng_2024_lens_review (membrane/biomechanics review), nishimoto_2003 (DNase II-beta), horwitz_1992 (alpha-crystallin chaperone) | refs-audit 2026-10-26: all 21 original refs confirmed real; cheng_2024 title fixed (PMID 39176256), wieghofer journal+DOI added, bishop PMID 15037566 added; li_2022_aqp0_adhesion added as precise AQP0 anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>LNS-005</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Lens</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Lens Nucleus (sutures, growth, transparency)</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>17 (development)</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>ch12: 422-425, 432-434 | nucleus = fetal/postnatal fibre junction (6.5 mm at birth); subdivisions: embryonic (primary fibres 6-7 wk / 18 mm), fetal (Y-sutures: 60-deg equatorial span -&gt; 30-deg branches, 6 branches, curvature pronounced), adult (9-point star: 8 arms, 20-deg meridional turn, half end anterior/posterior at 10-deg latitude; 4-star: 20-deg equator inserts &gt;75-deg suture); star position each ~15 yr, postnatal sutures offset (latticework, Fig 12.29); growth timeline: 18 mm AP elongation, 18-24 mm spherical, 26 mm secondary fibres equatorial widening, 65 mm zonule appears (no role in initial widening); first 2 decades sagittal plateau + nuclear width decrease + cortical increase (compaction, Forbes 1992 Fig 12.36; sagittal regression y=3.6234+1.1538e-2x+1.8593e-4x^2 R=0.875); from ~20 y sagittal resumes, equatorial negligible; +29 um/yr (Nielsen 1982, Brown 1973); specific gravity constant, nuclear density rises with age (Bours &amp; Fodisch 1986) - dehydration (slices) vs hydration up (Raman, Siebinga 1991) unresolved; slit zones (Fig 12.37): C1a postnatal, C1b, proto-C2,3,4, C3 ~7 yr increasing scattering lifelong, separates perinuclear C4 from superficial C2; zones move outward like ripple at constant distance from surface (Koretz 1984,1988); GRIN cortex-&gt;nucleus correlates protein content = refractive power + freedom from chromatic aberration (Phillipson 1969); pump-leak (Kinsey &amp; Reddy 1965, Fig 12.38): anterior Na/K-ATPase + Ca-ATPase + K in, posterior passive Na in/K out, gap junction equilibration</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>lens-nucleus.json</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff ch.12 scans 431-444.pdf pp.433-434 re-read this session)</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 39/39, 2026-10-26, incl. v1.1.0)</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>v1.1.0; created 2026-10-26 (nucleus + sutures + growth + transparency blocks). Clinical: at birth perfectly transparent; yellowing from UV 315-400 nm chromophores -&gt; visible+fluorescent pigments, possible retinal blue-light screening (Sliney &amp; Wolbarsht 1980); cortical pigment -&gt; perinuclear autofluorescence; brunescent senile nuclear cataract; insoluble protein rises (cross-linked crystallin aggregates); central metabolism negligible, no protein turnover (Harding &amp; Dilley 1976) -&gt; oxidative unfolding -&gt; sulphydryl -&gt; disulphide crosslinking; cataract opacity = zones of increased scattering (fibre irregularity, membrane degradation, aggregates) + swelling from ion/water disturbance (Harding 1991; Brown &amp; Bron 1996); suture planes = increased spherical aberration (Kuszak, Sivak &amp; Weeheim 1991); slit-lamp ageing/localisation of opacities; contusion opacity dating 2x growth speed | enrichment v1.1.0 APPLIED 2026-10-26: post-Wolff evidence merged into fields; refs: augusteyn_2010 (biphasic growth/nomenclature), jones_2005_grin, heys_2004 (nuclear stiffness &gt;1000x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>LNS-006</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Lens</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Ciliary Zonule (Zonule of Zinn)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>11 (ciliary body), 13 (vitreous)</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>ch12: 435-442 | fibres ciliary body -&gt; lens; ring triangular in meridional section, apex follows ciliary valleys over pars plana to ora serrata; fibrils = non-collagenous glycoprotein PAS+, elastin-like (size, tubular ultrastructure Raviola 1971, cross-reactivity, AA/peptide profiles, collagenase-resistant, trypsin/chymotrypsin-susceptible) = fibrillin cysteine-rich microfibril, template for elastin but never elasticized (like oxytalan); FBN1 15q21.1 (Lee 1991, Magenis 1991), Marfan = FBN1 mutations; fibrils 8-12 nm tubular, microperiodicity 12-14 nm (40-55 aggregated), beads 29 nm + ~4 filaments 3-6 nm, periodicity 30-57 nm (Wallace 1991); 4 topographic zones: pars orbicularis (pars plana, origin up to 1.5 mm from ora, bundles 2-5 fibrils into NP epithelium BM), zonular plexus (ciliary valleys, tension fibres anchor valley BM), zonular fork (angulation, 3 limbs), anterior/equatorial/posterior limbs; insertions: pre-equatorial double row bundles 5-10 um at ~1.5 mm, zone 0.3-0.4 mm, finger-like -&gt; zonular lamella (fibrils lost 1 mm central), anterior fibrils 0.07-0.5 um to depth 0.6-1.6 um, meridional 0.5-1.0 um wide -&gt; AP ribbing; equatorial sparse brush-like perpendicular 10-15 (to 60) um; posterior 2-3 layers over 0.4-0.5 mm extending 1.25 mm behind equator, depth ~2 um; attach up to 1 mm post / 1.5 mm ant of equator, crenated equator; hyaloid zonule single layer (Eisner 1973); hyalocapsular zonule = Wieger ligament (radial fibres); canals of Hannover (subdivided by equatorial fibres) + Petit; circumferential girdles (Eisner anterior ciliary girdle + posterior girdle, posterior bundle 1-2 mm anterior to ora = median vitreous tract insertion); aberrant fibres: traction tufts, meridional folds (Foos 1969); unit = flat ribbon 30-60 um wide, 6-10 per major ciliary process; Rohen 1979 accommodation schema (tension-fibre system at fork)</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>ciliary-zonule.json</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff ch.12 scan 445-453.pdf)</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 39/39, 2026-10-26, incl. v1.1.0)</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>v1.1.0; created 2026-10-26 (12.2 complete). Clinical: alpha-chymotrypsin zonulolysis in ICCE (Ley 1960); ICCE tears most of complex; ECCE dehiscences ~5% detected (Guzek 1987), more postmortem (Wilson 1987); PXF zonule 4x rupture risk in cataract surgery (Skuta 1987); Marfan ectopia lentis = FBN1; pigmentary glaucoma from posterior iris rub (Campbell 1979); ageing: fibres finer/sparser/rupture readily, attachments broaden + move central, zonule-free area 8 mm@20y -&gt; 6.5 mm 8th decade (-&gt;5.5) -&gt; capsulotomy planning (Farnsworth &amp; Shine 1979; Stark &amp; Streeten 1984), insertion-equatorial distance rises, circumlental space falls (Fig 12.47); Streeten 1992 mucoid diffusion-barrier speculation | enrichment v1.1.0 APPLIED 2026-10-26: post-Wolff evidence merged into fields; refs: genereviews_ectopia_lentis (ADAMTS10/17, ADAMTSL4, LTBP2), loeys_2010_ghent, bassnett_2020_zonule, aao_bcsc_lens (CTR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>VIT-001</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Vitreous</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Vitreous Body (gross appearances, spaces, Cloquet canal, topographic zones)</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>12 (lens/zonule relations)</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>ch13: 443-444, 446-447 | transparent colourless gel firmer than egg white; posterior 4/5 of globe; contact retina behind, ciliary body/zonule/lens in front; roughly spherical flattened anteriorly; patellar fossa + ciliary space of Berger; Wieger ring (ligamentum hyaloideocapsulare) 8-9 mm; union strong youth -&gt; weak by 6th decade permits intracapsular extraction; vitreous base 2 mm anterior over ciliary body / 4 mm posterior over peripheral retina (Fig 13.3); Cloquet canal 1-2 mm sinusuous lens-&gt;disc, area of Martegiani funnel in front of disc; primary vs secondary vitreous; topographic zones Fig 13.8 (preretinal 1 / intermediate 2 / retrolental 3); intraocular spaces catalog Fig 13.2 after Cibis 1965 (Berger, Petit, Hannover, hyaloideo-orbicular, indo-zonular, indocapsular); avascular adult, diffusion nutrition (Davson 1980); canal walls condensation (Mann 1927, Goldmann 1954, Busacca-Goldmann-Schiff-Wertheimer 1957), fenestrated sheaths of embryonic hyaloid artery media, cells + fine collagen (Balazs 1973); historical theories: alveolar Demours 1741, lamellar Zinn 1780, radial sector Hannover 1845, fibrillar Szent-Gyorgi 1917; Bowman 1849 fixative artefacts; slit-lamp era Gulstrand 1912 membranes, Koeppe 1917 fibres, Friedenwald &amp; Stiehler 1935 sheets; Eisner definitive account 1971-1982; birth homogeneous finely striated, no cortex/central distinction</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>vitreous.json</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff ch.13 scans 445-453.pdf p.9 + 454-463.pdf pp.1-4)</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 39/39, 2026-10-26, incl. v1.1.0)</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>v1.1.0; created 2026-10-26 (13.1 gross + topography + spaces + Cloquet). Registry note: comp_vitreous added to schemas/common/component-registry.json (row 37, has_3d_model No, unity vitreous_body) - registry previously had no vitreous component | enrichment v1.1.0 APPLIED 2026-10-26: post-Wolff evidence merged into fields; refs: uchino_2001_pvd (OCT stages), sebag_2004_anomalous_pvd, stalmans_2012_ocriplasmin</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>VIT-002</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Vitreous</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Vitreous Tracts (retrolental/coronary/median/preretinal + postnatal development)</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>12 (zonule), 14 (retina/ora)</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>ch13: 444-447 | fine sheet-like condensations radiating backwards from defined points on circumference of ciliary body and anterior retina -&gt; concentric onion-skin arrangement of adult vitreous; second postnatal development beginning anteriorly; RETROLENAL tract: inserts circular zone on lens capsule near hyaloideocapsular ligament, extends posteriorly, highly reflecting = membrana plicata of Vogt (Vogt 1941); CORONARY tract: from circular zone overlying posterior third of ciliary processes (coronary ligament), variable density fairly indistinct; MEDIAN tract: inserts at anterior margin of vitreous base mid-pars plana (median ligament), faint veil backwards; PRERETINAL tract: inserts at ora serrata, most strongly reflecting, least affected by age (Fig 13.7); Fig 13.9 schema TR/TC/TM/TP with LR/LC/LM/OS; gentle curvature youth -&gt; more sinuous+extensive with ageing, configuration depends on gravity (Nordmann &amp; Roth 1967; Eisner 1971); S-shaped course adult (descend behind lens, ascend centre, descend to disc); development timeline Fig 13.6: (a) late fetal hyaloid artery disc-&gt;lens + intravitreal limiting membrane of Dejeane, (b) infant artery+membrane gone regular fine striation, (c) adolescent anterior tracts begin posterior still infantile, (d) adult tracts reach posterior pole, (e) senile framework destruction liquid cavities + irregular strands, (f) senile PVD empties through gap retrovitreal collapse (Eisner in Duane &amp; Jaeger 1987); optical dissections Fig 13.7: 32-wk hyaloid artery + Bergmeister papilla remnants, 7-mo tiny remnants + prepapillary channel no tracts, 14-y anterior cortex delineated, 70-y tracts near posterior pole, destruction from 31-y cavities, 75-y PVD collapsed strands intravitreal-&gt;retrovitreal; transvitreal channels overlie disc/fovea/vessels = vitreous synthesis variation during growth (Eisner 1973a,b, 1975, 1978; Eisner &amp; van den Zypen 1981); central density decreases cortex retains higher density (Eisner &amp; Bachmann 1974a-d); interspecies: cat highest central density, cattle/sheep homogeneous, horse low; liquefaction + fibrillar degeneration from adolescence breaks tract pattern</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>vitreous-tracts.json</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff ch.13 scans 454-463.pdf pp.2-4)</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 39/39, 2026-10-26, incl. v1.1.0)</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>v1.1.0; created 2026-10-26 (tracts + ligaments + development timeline). Clinical: onion-skin pattern = normal biomicroscopic architecture; breakdown substrate of senile PVD; preretinal tract least affected = enduring base strength; developmental remnants (hyaloid artery, Bergmeister papilla, prepapillary channel) vs pathology; fluid central vitreous passes through break posteriorly, posterior hyaloid forwards (Eisner 1982; Sebag &amp; Balazs 1984) | enrichment v1.1.0 APPLIED 2026-10-26: post-Wolff evidence merged into fields; refs: uchino_2001_pvd, johnson_2010_pvd</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>VIT-003</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Vitreous</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Vitreous Cortex (anterior/posterior hyaloid, vitreous base, peripapillary/perimacular attachments)</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>14 (ILM/Muller cells), 12 (zonule relations)</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>ch13: 447-450, 452 | MICROSCOPIC STRUCTURE 13.2 components: cortex (anterior hyaloid, vitreous base, posterior hyaloid, peripapillary+perimacular attachments), central vitreous, vitreous cells; CORTEX = clinically dense broad zone up to 0.2-0.3 mm adjoining retina (Fig 13.12); microscopically outer 100-200 um, condensation of fibrils+cells+GAG (Balazs 1961); surface condensation = fragile envelope, not distinct hyaloid membrane; absent just anterior to base (zonular cleft of Salzmann) + area of Martegiani; Salzmann anterior/posterior limiting layers = anterior/posterior hyaloid to margins of anatomical base; Eisner posterior/anterior cortex + intermediate/retrolenticular central subdivisions (1982); ANTERIOR HYALOID: from anterior margin of base at ora, epiciliary portion to hyaloideocapsular ligament, retrolental portion thinned; floats freely in some adults (Eisner 1973a,b); after extracapsular extraction seen more clearly; hyalociliary zonule fibres to valleys between ciliary processes + 3 circular zonular sets (Graf Spee 1902): retrolental ligament = lig. hyaloideocapsulare, coronary ligament across posterior third of ciliary processes, median ligament at mid pars plana; fibres interwoven into anterior cortex, radial fibres to ciliary body/lens (Daicker 1972); anterior cortex compacted lamellae parallel with pars plana, mesh-like (Fine &amp; Tousimis 1961; Faulborn &amp; Bowald 1982); VITREOUS BASE: band 2.0 mm anterior ora -&gt; 2-4 mm behind; fibrils most densely packed, adult insert throughout width (Sebag, Balazs &amp; Flood 1984); anterior blend with basal lamina of non-pigmented pars plana epithelium, behind with ILM; tapering bundles right-angles to retinal surface, finer anteriorly fanning to lens; base fibrils wider ~45 nm; most established portion = narrow band over ora; infancy just posterior to ora, broadens with age (Hogan 1963; Daicker 1972), straight temporally/wandering nasally; racial: more posterior in African and Chinese; POSTERIOR HYALOID: fibrils curve backwards along inner retina, blend with ILM posterior to equator, more readily identified in fetal eyes; PERIPAPILLARY cortex: firm union to marginal retina 10 um wide at disc edge where Muller fibres+ILM end; PERIMACULAR similar but less dense; both more developed in young eyes (Fig 13.15 premacular PM + prepapillary PP holes); fibrils ~12 nm insert into ILM/Muller basal lamina; firm bond at base/disc/macula/vessels strong in youth weakens with age, loose elsewhere; young eyes Muller cell membrane breaks before attachment (Sebag 1989); ILM thickness 20-100 nm -&gt; 3 um with age (Foos 1972), barrier to macromolecules &gt;=7 nm; interrupted at pars plana/ciliary processes = direct fibril-epithelium contact; breaks increase with age, fragments in adult cortex (Rentsch &amp; van der Zypen 1971); sublaminar space fibrils at attachment plaques (Fig 13.13); traction on base -&gt; retinal tear -&gt; detachment forerunner (Chaine, Jebay &amp; Coscas 1983); aging base crypts between Muller foot plates, fibres perforate ILM fill crypt (p.458, Fig 14.7)</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>vitreous-cortex.json</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff ch.13 scans 454-463.pdf pp.4-7)</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 39/39, 2026-10-26, incl. v1.1.0)</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>v1.1.0; created 2026-10-26 (13.2 microscopic structure: cortex + 4 attachment zones + vitreoretinal junction). Clinical: strength map (firm base/disc/macula/vessels vs loose elsewhere) = substrate of traction pathology; age weakening = PVD basis | enrichment v1.1.0 APPLIED 2026-10-26: post-Wolff evidence merged into fields; refs: uchino_2001_pvd, johnson_2010_pvd, sebag_2004_anomalous_pvd (vitreoschisis)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>VIT-004</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Vitreous</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Hyalocytes / Vitreous Cells (mononuclear phagocytes of the cortical gel)</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>14 (RPE after retinal damage)</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>ch13: 451, 452 | VITREOUS CELLS (OR HYALOCYTES): cells present ONLY in cortex adjacent to retina and ciliary body; central vitreous + cortex adjacent to lens/posterior chamber completely cell-free in normal adult eyes; most prominent at vitreous base, over optic nerve head, in relation to retinal vessels; vast majority = mononuclear phagocytes (macrophages called hyalocytes); some fibrocytes + various glial cells also found (Figs 13.17, 13.18); HYALOCYTES: phagocytic cells, many lysosomes, some phagosomes, prominent Golgi complex; affinity for neutral red; intense red autofluorescence; large electron-dense inclusions; phagocytic properties demonstrated in vivo AND in vitro; hydrolytic enzymes in lysosomes; capable of synthesizing hyaluronic acid; normal vitreous = resting population in cortex, usually NOT in contact with basal lamina; Fig 13.17 phase contrast flat mount (11-year-old post mortem, Sebag 1989): mononuclear cells in single layer within cortex, round appearance, pseudopodia in some; Fig 13.18 EM posterior retinal surface: migratory cell with pseudopodia + vacuoles / round cell rich in intracytoplasmic filaments (van der Zypen); INFLAMMATION: numbers increase, found in central vitreous, penetrate basal lamina in passage to/from retina or ciliary body; macrophage population expanded by other monocytic-origin cells or, after retinal damage, by retinal pigment epithelial cells (Hogan, Alvarado &amp; Weddell 1971; Balazs 1973); HA synthesis links to gel maintenance + transparency; scavenging role in normally cell-free cavity</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>hyalocytes.json</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff ch.13 scans 454-463.pdf pp.8-9)</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 39/39, 2026-10-26, incl. v1.1.0)</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>v1.1.0; created 2026-10-26 (13.2 vitreous cells: hyalocytes + population composition + inflammation response). Clinical: cellular basis of vitritis; hyalocyte mobilization through basal lamina; RPE recruitment after retinal damage | enrichment v1.1.0 APPLIED 2026-10-26: post-Wolff evidence merged into fields; refs: wieghofer_2022_hyalocytes (myeloid origin), boneva_2020_hyalocytes (transcriptional identity)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>VIT-005</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Vitreous</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Vitreous Composition (water 99%, hyaluronic acid, type II collagen, aqueous-like solutes)</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>12 (lens capsule collagen contrast)</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>ch13: 452 (+450 Fig 13.16) | COMPOSITION 13.3: vitreous 99% water, volume ~4.0 ml; liquid phase contains hyaluronic acid = high molecular weight proteoglycan (33-61 kDa) responsible for characteristic high viscosity; concentration in human vitreous 0.03-0.1% (Balazs 1973); HA molecular diameter 0.1-0.5 um; fine fibrillar collagen relatively resistant to trypsin and alpha-chymotrypsin, digested by pepsin and collagenase, DIFFERENT from ocular coats or lens capsule; biochemically type II collagen, moderate sugar content lower than basement membrane collagens; types IX and XI also present; fibrillar diameter 6-16 nm, microperiodicity 22 nm; 64 nm periodicity with phosphotungstic acid staining + shadow casting (Schwarz 1956; Balazs 1961; Fine &amp; Tousimis 1961; Hogan 1963; Swan 1980); fibrils coated with glycosaminoglycan, stainable with ruthenium red, removed with hyaluronidase (Brini, Porte &amp; Stoeckel 1968); composition otherwise similar to aqueous apart from quantitative and regional differences; free diffusion of water between vitreous and aqueous compartments (Davson 1980); movement of large solute molecules restricted by gel-like structure -&gt; influences distribution, delivery and removal of drugs and other materials; Fig 13.16 Balazs schematic: collagen filament 10 nm + HA coils 150 nm, repeats over ~1200 nm span, liquid vitreous between fibres; HA maintains physical separation of collagen filaments = optical transparency</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>vitreous-composition.json</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff ch.13 scan 454-463.pdf pp.9-10)</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 39/39, 2026-10-26, incl. v1.1.0)</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>v1.1.0; created 2026-10-26 (13.3 composition). Clinical: gel restricts large solutes = basis of intravitreal drug behaviour; type II collagen enzymatic identity (trypsin/alpha-chymotrypsin resistant, pepsin/collagenase digested) distinguishes vitreous from coats/capsule | enrichment v1.1.0 APPLIED 2026-10-26: post-Wolff evidence merged into fields; refs: bishop_2004_collagen (heterotypic fibrils II+V/XI+IX), legoff_2008_vitreous (HA megadalton reconciliation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>VIT-006</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Vitreous</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Vitreous Ageing and Detachment (syneresis, collapse, PVD mechanism, retinal tear risk)</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>14 (retinal tears/holes, ILM)</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>ch13: 452-453 | AGEING AND VITREOUS DETACHMENT 13.4: young eye relatively empty optically on slit-lamp; with age veil-like light scattering undulating with eye movements = presumed gel structure alteration, NOT visibility of collagen fibrils (molecular dimensions); old age or younger MYOPIC eye: breakdown in structure = increased scattering + optically empty spaces (syneresis) (Figs 13.19, 13.20); altered gel may collapse so outer surface pulls away from internal coats = vitreous detachment; facilitated by age weakening of adhesion between vitreous and external structures; detachment spectrum: may merely SPLIT the internal limiting membrane at attachment points / SEPARATE vitreous from ILM / SPLIT the cortical vitreous / at times TEAR the retina itself -&gt; retinal hole -&gt; precursor of retinal detachment (Balazs 1973; Foos 1975; Daicker, Guggenheim &amp; Guyat 1977); vitreous detachment = NORMAL consequence of ageing, frequent in otherwise normal eyes in old age (Jokl 1927); usually precipitated by hole in posterior vitreous face when vitreous separates from normally strong attachment around macula or optic disc; fluid central vitreous passes posteriorly through hole while posterior hyaloid moves forwards (Eisner 1982; Sebag &amp; Balazs 1984); Fig 13.19 79-year-old dissection: fibrillar structure well seen dark-field, base/ora intact; Fig 13.20 88-year-old: overall collapsed (syneresis), fibres tortuous aggregated thickened, large lacunae of liquid vitreous peripherally (Sebag)</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>vitreous-detachment.json</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff ch.13 scan 454-463.pdf pp.9-10)</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 39/39, 2026-10-26, incl. v1.1.0)</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>v1.1.0; created 2026-10-26 (13.4 ageing + detachment). Clinical: PVD normal ageing event (Jokl 1927); 4-plane separation spectrum explains RD precursor risk; myopia = earlier breakdown | enrichment v1.1.0 APPLIED 2026-10-26: post-Wolff evidence merged into fields; refs: uchino_2001_pvd, johnson_2010_pvd, hikichi_2004_fellow_eye (65% within 2y), sebag_2004_anomalous_pvd, stalmans_2012_ocriplasmin</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Enrich optic nerve and sclera knowledge cards
</commit_message>
<xml_diff>
--- a/Anatomy_Extraction_Master_Tracker_v2.xlsx
+++ b/Anatomy_Extraction_Master_Tracker_v2.xlsx
@@ -3081,7 +3081,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>ch7: 269-278 (episclera 270-271, dimensions 272, apertures 272-274, organization 275-276, blood/nerve 276-277, ageing 277-278) | ch17: 628-632 (17.3 SCLERA opening: neural crest origin, &lt;6.5 wks 8-9 layers, demarcation mid-7th wk 15 layers, 9th wk 48nm, 30-&gt;50 layers, IGF-II/myopia) [16.pdf + full-book scan]</t>
+          <t>ch7: 269-278 (episclera 270-271, dimensions 272, apertures 272-274, organization 275-276, blood/nerve 276-277, ageing 277-278) | ch17: 628-632 (17.3 SCLERA opening: neural crest origin, &lt;6.5 wks 8-9 layers, demarcation mid-7th wk 15 layers, 9th wk 48nm, 30-&gt;50 layers, IGF-II/myopia) [16.pdf + full-book scan] | ch7 add: 274 (nerve loop of Axenfeld), 275 (Kokott force interpretation)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -3151,7 +3151,7 @@
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>v1.0.0; created 2026-10-23 from Wolff Ch.7 pp.269-278 | v1.1.0+v1.2.0 dev enrichment 2026-10-23</t>
+          <t>v1.0.0; created 2026-10-23 from Wolff Ch.7 pp.269-278 | v1.1.0+v1.2.0 dev enrichment 2026-10-23 | v1.3.0 (2026-10-27) ch7 text re-delivery dedupe pass: 269-278 verified largely covered; NEW - nerve loop of Axenfeld (12% of eyes, bilateral 1%, multiple occasionally; smooth glistening grey domes 1-2mm, Stevenson 1963) appended to innervation (p.274) + Kokott biomechanical interpretation (bundle array from IOP + muscle pull, femoral-neck trabeculae analogy, peripapillary circular 4mm, balloon-net posterior pattern) appended to histology (p.275); keywords +4; validate 27/27 + pytest green</t>
         </is>
       </c>
     </row>
@@ -3258,7 +3258,7 @@
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>v1.0.0; ciliary injection, sub-Tenon plane, episcleritis | v1.1.0 dev enrichment 2026-10-23</t>
+          <t>v1.0.0; ciliary injection, sub-Tenon plane, episcleritis | v1.1.0 dev enrichment 2026-10-23 | v1.2.0 (2026-10-27) ch8 text: formal three-zone limbus division (deep = TM + Schlemm's canal / mid = transitional corneoscleral stroma + intrascleral venous plexus / superficial = episclera + Tenon + conjunctival stroma + limbal epithelium) + limbus dimensions 1.5mm (~2mm vertical) appended to location (pp.279-280); keywords +4; validate 27/27</t>
         </is>
       </c>
     </row>
@@ -3472,7 +3472,7 @@
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>v1.0.0; SSC myofibroblasts; miotic mechanism; gonioscopic landmark | v1.1.0 dev enrichment 2026-10-23</t>
+          <t>v1.0.0; SSC myofibroblasts; miotic mechanism; gonioscopic landmark | v1.1.0 dev enrichment 2026-10-23 | v1.2.0 (2026-10-27) ch8 text: peptidergic/nitrergic innervation (NPY/SP/CGRP/VIP/NO immunoreactive, acetylcholinesterase-negative; VIP+nitrergic likely pterygopalatine parasympathetic, SP+CGRP mostly trigeminal sensory; outflow-resistance modulation via tendon-like contacts; VIP/CGRP/nitrovasodilators raise outflow facility in cynomolgous monkey, Tamm 1995b) appended to innervation (pp.284-285); keywords +6; validate 27/27</t>
         </is>
       </c>
     </row>
@@ -3616,7 +3616,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>ch15: 503-508, 528-534 (disc area 0.86-5.54 mm2 mean 2.69±0.7 + macrodiscs &gt;4.09/microdiscs &lt;1.29 (Jonas/Gusek/Naumann 1988, 1991) + Table 15.1 full metrics 505; lamina area 2.88±0.84 mm2 + pore count 227±36 (Jonas 1991) + cup metrics + rim broadest inferior-&gt;superior-&gt;nasal-&gt;temporal, narrowest temporal horizontal in 99.2% 506; cup/disc ratio median 0.3, vertical lower in 93.2%, asymmetry &gt;0.2 diagnostic; parapapillary zones alpha 84.4%/beta 15.2% + POAG alpha 0.65/beta 0.79 507; RNFL visibility order + axon loss 4-5000/yr 508; ONH watershed + zonal arterial supply + venous drainage + opticociliary veins 528-534) [scans 13.pdf+14.pdf] | v1.1.0 pages: 530, 533, 534-535 + 530-560.pdf/586.pdf</t>
+          <t>ch15: 503-508, 528-534 (disc area 0.86-5.54 mm2 mean 2.69±0.7 + macrodiscs &gt;4.09/microdiscs &lt;1.29 (Jonas/Gusek/Naumann 1988, 1991) + Table 15.1 full metrics 505; lamina area 2.88±0.84 mm2 + pore count 227±36 (Jonas 1991) + cup metrics + rim broadest inferior-&gt;superior-&gt;nasal-&gt;temporal, narrowest temporal horizontal in 99.2% 506; cup/disc ratio median 0.3, vertical lower in 93.2%, asymmetry &gt;0.2 diagnostic; parapapillary zones alpha 84.4%/beta 15.2% + POAG alpha 0.65/beta 0.79 507; RNFL visibility order + axon loss 4-5000/yr 508; ONH watershed + zonal arterial supply + venous drainage + opticociliary veins 528-534) [scans 13.pdf+14.pdf] | v1.1.0 pages: 530, 533, 534-535 + 530-560.pdf/586.pdf | v1.2.0 pages: ch15: 494-495 (Anderson 1969 Fig 15.8: prelaminar astrocytic tubes with perpendicular astrocytes + intratubular capillaries; laminar fascicle astrocyte layer + connective-tissue mantle; postlaminar oligodendrocyte columns; border tissue of Jacoby cuff -&gt; intermediary tissue of Kuhnt forwards, glial mantle backwards)</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -3686,7 +3686,7 @@
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)] | v1.1.0 enrichment 2026-10-24: from batch-3 pages (525, 535-545, 586-590): circle of Zinn-Haller frequency dispute (Olver 1990 frequently present vs Hayreh small proportion; often incomplete Levitzky &amp; Henkind 1969; ABSENT in sub-human primates Hayreh 1964; horizontal-ellipse intrascleral anastomosis of medial+lateral paraoptic SPCA branches; paraoptic replacements when absent) + positional variants (apposed/distant/anterior intrascleral/posterior extrascleral; axial position on SEM) appended to blood_supply; marginal tissue of Kuhnt glial 'gasket' tight junctions appended to histology (Tso/Shih/McLean 1975); incomplete ONH blood-brain barrier with HRP tracer route choroid-&gt;prelaminar-&gt;lamina septa-&gt;retrolaminar + implications for optic pits and papilloedema appended to clinical (pp.534-535); bilingual keywords extended; validate 27/27 + pytest 10+14 green</t>
+          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)] | v1.1.0 enrichment 2026-10-24: from batch-3 pages (525, 535-545, 586-590): circle of Zinn-Haller frequency dispute (Olver 1990 frequently present vs Hayreh small proportion; often incomplete Levitzky &amp; Henkind 1969; ABSENT in sub-human primates Hayreh 1964; horizontal-ellipse intrascleral anastomosis of medial+lateral paraoptic SPCA branches; paraoptic replacements when absent) + positional variants (apposed/distant/anterior intrascleral/posterior extrascleral; axial position on SEM) appended to blood_supply; marginal tissue of Kuhnt glial 'gasket' tight junctions appended to histology (Tso/Shih/McLean 1975); incomplete ONH blood-brain barrier with HRP tracer route choroid-&gt;prelaminar-&gt;lamina septa-&gt;retrolaminar + implications for optic pits and papilloedema appended to clinical (pp.534-535); bilingual keywords extended; validate 27/27 + pytest 10+14 green | v1.2.0 (2026-10-26) batch-5: owner text printed 494 (+495 continuation verified visually from scan render) - prelaminar astrocytic-tube architecture (bundles + perpendicular astrocytes, capillaries within tubes), peripheral astrocyte cuff = border tissue of Jacoby continuing forwards as intermediary tissue of Kuhnt and backwards in continuity with glial mantle deep to pia, laminar astrocyte layer + mantle of connective tissue (collagen/elastic/fibroblasts/capillaries) thinner than prelaminar, postlaminar myelination with columns of oligodendrocytes + few astrocytes, glial separation rule (Anderson/Hoyt/Hogan 1967) with CRA-adventitia exception (Ikui 1964) appended to layers[1..3]; keywords +10; validate 27/27 + pytest green. | 2026-10-26 restore: v1.2.0 batch-5 card text re-applied after local workspace rollback lost the files (reconstructed from these tracker notes + session record - content equivalent, sources identical); validate 27/27 + pytest green</t>
         </is>
       </c>
     </row>
@@ -3830,7 +3830,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>ch15: 499, 515-518, 521 (septa invade with vessels ~4th month; 6-9 primary septa into sectors + dichotomous secondary septa; interseptal spaces rounded in human vs polygonal in other mammals 517; septa = tubes around fascicles, fenestrated; trabecula central vessel with muscular/elastic layers; astrocyte feet + basal lamina + invaginations 120-150 um (Anderson &amp; Hoyt 1969); astrocytes abut capillaries directly in chiasma 521; triangular glial septum separates ventromedial (crossing) from dorsolateral, marks start of decussation 518; support deficiency superior/inferior -&gt; early glaucomatous bowing (Quigley) 499) [scans 13.pdf] | v1.1.0 pages: 525, 529 + 530-560.pdf/586.pdf</t>
+          <t>ch15: 499, 515-518, 521 (septa invade with vessels ~4th month; 6-9 primary septa into sectors + dichotomous secondary septa; interseptal spaces rounded in human vs polygonal in other mammals 517; septa = tubes around fascicles, fenestrated; trabecula central vessel with muscular/elastic layers; astrocyte feet + basal lamina + invaginations 120-150 um (Anderson &amp; Hoyt 1969); astrocytes abut capillaries directly in chiasma 521; triangular glial septum separates ventromedial (crossing) from dorsolateral, marks start of decussation 518; support deficiency superior/inferior -&gt; early glaucomatous bowing (Quigley) 499) [scans 13.pdf] | v1.1.0 pages: 525, 529 + 530-560.pdf/586.pdf | v1.2.0 pages: ch15: 494 (Anderson 1969: laminar/postlaminar astrocyte layer thinner than prelaminar; oligodendrocyte columns in myelinated fascicles; lamina-cribrosa connective tissue continuous posteriorly with pial septae)</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -3900,7 +3900,7 @@
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)] | v1.1.0 enrichment 2026-10-24: from batch-3 pages: pial plexus centripetal branches each within a glial-coated connective-tissue core (p.525) + CRA intraneural branches anastomosing with the septal arteriolar/capillary system (p.529) + full intraseptal microvasculature account (large precapillaries/capillaries confined to septae in transverse and longitudinal polygonal units; extensive anastomosis, size non-uniformity, numbers increasing near posterior laminal bowing; anterior anastomosis with laminar vessels, posterior with intraorbital septal system — Lieberman/Maumenee/Green 1976) appended to blood_supply; bilingual keywords extended; validate 27/27 + pytest 10+14 green</t>
+          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)] | v1.1.0 enrichment 2026-10-24: from batch-3 pages: pial plexus centripetal branches each within a glial-coated connective-tissue core (p.525) + CRA intraneural branches anastomosing with the septal arteriolar/capillary system (p.529) + full intraseptal microvasculature account (large precapillaries/capillaries confined to septae in transverse and longitudinal polygonal units; extensive anastomosis, size non-uniformity, numbers increasing near posterior laminal bowing; anterior anastomosis with laminar vessels, posterior with intraorbital septal system — Lieberman/Maumenee/Green 1976) appended to blood_supply; bilingual keywords extended; validate 27/27 + pytest 10+14 green | v1.2.0 (2026-10-26) batch-5: owner text printed 494 (Fig 15.8) - laminar/postlaminar septal architecture appended to histology_summary: astrocytes separating fascicles thinner than prelaminar, myelinated fascicles contain oligodendrocyte columns, connective tissue of lamina cribrosa continuous posteriorly with pial septae; keywords +5; validate 27/27 + pytest green. | 2026-10-26 restore: v1.2.0 batch-5 card text re-applied after local workspace rollback lost the files (reconstructed from these tracker notes + session record - content equivalent, sources identical); validate 27/27 + pytest green</t>
         </is>
       </c>
     </row>
@@ -3937,7 +3937,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>ch15: 521-524, 527-534 (pial network double system + septal distribution exact = vessels 521; perichiasmal artery largest intracranial supply, origin superior hypophyseal (Hayreh 1963/Steele &amp; Blunt 1956) vs Dawson 1958 ophthalmic 522; intracanalicular OA sole supply, poor pial network vulnerable to shearing in skull fracture 524; intraorbital: CRA enters 5-15.5 mm behind globe, proximal centripetal vs distal axial, 3 sources, direct branches reach pia in 75% when OA crosses above (82-85% of cases) 524; venous drainage: pial veins + central retinal vein(s) (embryonic 2 channels beside hyaloid artery 3rd month; exit same aspect in 42%, vein anterior to artery in 81% (Fry 1930); intravaginal course 3.8-8 mm) + posterior central vein 527; cavernous sinus blockage does not block CRV flow 528; laminar circle of Zinn (1755)/Haller (1754) branches 1-4 + interfacial precapillaries vulnerable to raised IOP -&gt; disc haemorrhages (Ruskell 1984) 531; prelaminar scleral SPCA vs recurrent choroidal (only 10% choroidal origin, Lieberman 1976) + microvascular cuff 534; SNFL 5 supplies with CRA major 534; BBB incomplete at ONH (pars choroidalis) 534) [scans 13.pdf+14.pdf] | v1.1.0 pages: 525-526, 530, 533, 541, 543 + 530-560.pdf/586.pdf</t>
+          <t>ch15: 521-524, 527-534 (pial network double system + septal distribution exact = vessels 521; perichiasmal artery largest intracranial supply, origin superior hypophyseal (Hayreh 1963/Steele &amp; Blunt 1956) vs Dawson 1958 ophthalmic 522; intracanalicular OA sole supply, poor pial network vulnerable to shearing in skull fracture 524; intraorbital: CRA enters 5-15.5 mm behind globe, proximal centripetal vs distal axial, 3 sources, direct branches reach pia in 75% when OA crosses above (82-85% of cases) 524; venous drainage: pial veins + central retinal vein(s) (embryonic 2 channels beside hyaloid artery 3rd month; exit same aspect in 42%, vein anterior to artery in 81% (Fry 1930); intravaginal course 3.8-8 mm) + posterior central vein 527; cavernous sinus blockage does not block CRV flow 528; laminar circle of Zinn (1755)/Haller (1754) branches 1-4 + interfacial precapillaries vulnerable to raised IOP -&gt; disc haemorrhages (Ruskell 1984) 531; prelaminar scleral SPCA vs recurrent choroidal (only 10% choroidal origin, Lieberman 1976) + microvascular cuff 534; SNFL 5 supplies with CRA major 534; BBB incomplete at ONH (pars choroidalis) 534) [scans 13.pdf+14.pdf] | v1.1.0 pages: 525-526, 530, 533, 541, 543 + 530-560.pdf/586.pdf | v1.2.0 pages: ch11: 386 (Fig 11.13 Olver 1990 cast: temporal+medial SPCA bundles supply choroid AND retrolaminar nerve; paraoptic branches -&gt; circle of Zinn-Haller -&gt; pial branches to retrolaminar nerve + recurrent choroidal to peripapillary and peripheral vertical meridional choroid; triangular/trapezoid SPCA territories) | v1.3.0 sources: StatPearls NBK507907 + NBK542287 read in full | ch3: 87-88, 94</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -4007,7 +4007,7 @@
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)] | v1.1.0 enrichment 2026-10-24: batch-3 pages mined heavily: intraorbital layers block extended with the long-awaited p.525 material (pial plexus tortuous anastomoses reinforced at nerve-globe junction by scleral SPCA/circle of Zinn; centripetal branches within glial-coated cores; CRA origin variants relative to ophthalmic artery crossing; CRA course - dura piercing 5-15.5 mm inferomedially, intravaginal 0.9-2.5 mm in subarachnoid space, vertical entry + right-angled bend, ~5/3/8 intraorbital/intravaginal/intraneural branches; Hayreh 1963 stats - branches in all but 3.1%, none to lamina cribrosa, lacking intraorbital 47.8%/intravaginal 5.3%/intraneural 25%; collaterals superior/inferior per OA crossing, lateral rare vs Hughes 1954; CRA pial territory always inferior, superior least) + blood_supply extended with CRA wall structure (intima duplicated BM thickening with age; IEL irregular, disappears at lamina, absent from retinal arteries; media ~6 layers; adventitia continuous with septa) + GCA rule (only IEL-bearing vessels affected; retinal arteries spared - Cogan 1974) + Zinn-Haller frequency/form/position (pp.530-533) + chiasmal arterial supply (rich collateral anastomosis; Wollschlaeger 1971 630 specimens dorsal A1/ventral ICA-ACOMM with A2 contribution always per Perlmutter &amp; Rhoton 1976, no PCOMM/PCA/basilar contributions, superior hypophyseal + MCA feeders, dorsal/ventral classification) (pp.541-543) + GCA fact added to clinical; bilingual keywords extended; validate 27/27 + pytest 10+14 green</t>
+          <t>v1.0.0; created 2026-10-24 from Wolff Ch.15 "The Visual Pathway - Optic Nerve" printed pp.495-534 [scans 13.pdf (printed 495-524) + 14.pdf (printed 527-534)] | v1.1.0 enrichment 2026-10-24: batch-3 pages mined heavily: intraorbital layers block extended with the long-awaited p.525 material (pial plexus tortuous anastomoses reinforced at nerve-globe junction by scleral SPCA/circle of Zinn; centripetal branches within glial-coated cores; CRA origin variants relative to ophthalmic artery crossing; CRA course - dura piercing 5-15.5 mm inferomedially, intravaginal 0.9-2.5 mm in subarachnoid space, vertical entry + right-angled bend, ~5/3/8 intraorbital/intravaginal/intraneural branches; Hayreh 1963 stats - branches in all but 3.1%, none to lamina cribrosa, lacking intraorbital 47.8%/intravaginal 5.3%/intraneural 25%; collaterals superior/inferior per OA crossing, lateral rare vs Hughes 1954; CRA pial territory always inferior, superior least) + blood_supply extended with CRA wall structure (intima duplicated BM thickening with age; IEL irregular, disappears at lamina, absent from retinal arteries; media ~6 layers; adventitia continuous with septa) + GCA rule (only IEL-bearing vessels affected; retinal arteries spared - Cogan 1974) + Zinn-Haller frequency/form/position (pp.530-533) + chiasmal arterial supply (rich collateral anastomosis; Wollschlaeger 1971 630 specimens dorsal A1/ventral ICA-ACOMM with A2 contribution always per Perlmutter &amp; Rhoton 1976, no PCOMM/PCA/basilar contributions, superior hypophyseal + MCA feeders, dorsal/ventral classification) (pp.541-543) + GCA fact added to clinical; bilingual keywords extended; validate 27/27 + pytest 10+14 green | v1.2.0 (2026-10-26) batch-5: owner text printed 386 (ch.11 Fig 11.13) - Olver/Spalton/McCartney 1990 posterior-pole vascular cast appended to blood_supply: SPCA dual supply (choroid + retrolaminar nerve), Zinn-Haller outflow to pial and recurrent choroidal branches incl. peripheral vertical meridional choroid, triangular/trapezoid choroidal territories; keywords +7; pages screened not cited: 30 (eyelids), 192 (trigeminal ganglion, ON in Fig 5.16 label only), 283 (Schlemm/sulcus), 361 (ciliary ageing), 403 (ciliary vessels), 665-693 bibliography (no anatomical facts; relevant ON literature already cited in-text); validate 27/27 + pytest green. | batch-6 screening (2026-10-26): owner text printed 390 (Fig 11.13 contd q-t - choroidal venous casts: collecting venules, vortex tributaries, venulo-venular anastomoses), 396 (choriocapillaris ultrastructure - 60-80nm fenestrations, pericytes, leaky discontinuous zonulae occludentes, Bruch's membrane 5 layers), 666 + 675 (bibliography; confirms primary refs already cited in-card: Anderson 1969b 82:800, Anderson &amp; Braverman 1976, Anderson/Hoyt/Hogan 1967) - choroid-domain or bibliography content, no optic-nerve facts, not cited per scope rule; material flagged for a future Choroid category. Pages 718-719/722-723 NOT received (second message truncation) - outstanding. | v1.3.0 (2026-10-26) StatPearls round: teaching-source corroboration appended to blood_supply (ophthalmic artery = first branch of ICA arising just distal to cavernous sinus; within the optic canal it courses inferior and lateral to the nerve before its intraorbital crossing; circle of Willis encircles the opto-chiasmatic region with branches perfusing intracranial nerve and chiasm; 25/25 quote checks); keywords +4; validate 27/27 green. Cards ON-002/ON-004 unchanged - corroborating StatPearls facts already covered by Wolff citations.  | v1.4.0 (2026-10-27) Wolff ch3 owner text (87-88, 94): OA origin medial convex side of 5th ICA bend, medial to anterior clinoid, inferior to nerve mid-point; initial limb 1-2mm below nerve -&gt; right-angle bend under medial side -&gt; long limb anterolateral to inferolateral surface; lateral-margin angle obtuse 120-135deg in 56% / right 40% / acute 4% (Hayreh 1972); canal: leaves subdural to enter sheath between fused dura-periosteum, leaves near orbital end, calibre diminished; crosses OVER nerve 82.6% vs under 17.4% (Hayreh &amp; Dass 1962b); CRA first branch when over, lateral PC when under; 14-branch order; fetal derivation (dorsal ophthalmic -&gt; trunk+lateral PC+CRA; ventral -&gt; medial PC; stapedial -&gt; rest, Hayreh 1963); PC arteries 2-4 trunks below nerve -&gt; 10-20 branches; ACA supplies upper chiasma + intracranial optic nerve (p.94); keywords +10; validate 27/27 + pytest green</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add and enrich Choroid knowledge cards
</commit_message>
<xml_diff>
--- a/Anatomy_Extraction_Master_Tracker_v2.xlsx
+++ b/Anatomy_Extraction_Master_Tracker_v2.xlsx
@@ -1052,7 +1052,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U40"/>
+  <dimension ref="A1:U47"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="5"/>
   <sheetData>
     <row r="1">
@@ -5292,6 +5292,755 @@
       <c r="U40" t="inlineStr">
         <is>
           <t>v1.1.0; created 2026-10-26 (13.4 ageing + detachment). Clinical: PVD normal ageing event (Jokl 1927); 4-plane separation spectrum explains RD precursor risk; myopia = earlier breakdown | enrichment v1.1.0 APPLIED 2026-10-26: post-Wolff evidence merged into fields; refs: uchino_2001_pvd, johnson_2010_pvd, hikichi_2004_fellow_eye (65% within 2y), sebag_2004_anomalous_pvd, stalmans_2012_ocriplasmin</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>CHO-001</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Choroid</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Choroid (gross anatomy, circulation physiology, ageing/glaucoma, development)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>2,3,7,8,14,15,16,17</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>ch11: 371-410; ch2: 212-228; ch3: 88,101; ch7: 276-277; ch8: 302; ch15: 500-502 | pia-arachnoid homologue + cavernous-tissue look (376); fixed 100/220um vs in-vivo sonar 500-1000um Coleman &amp; Lizzi 1979 (376); flow 10:1 human / 20x monkey, no autoregulation (407-408); thinner in high myopia + congenital/chronic glaucoma (376); ageing Ramrattan 1994 + glaucoma Kubota 1993 (410); development ch17 637-640; osmotic anchoring 15mmHg + thermoregulation (408)</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>choroid.json</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff ch.11 full 371-410 + cross-chapters 2/3/7/8/15/17)</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 46/46, 2026-10-27)</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>v1.0.0; created 2026-10-27 from complete ch11 (371-410) + cross-chapter harvest. component_ids [comp_sclera, comp_retina] because choroid has no object in the model registry (intermediate coat between the two). 8/8 fields documented, 1,343 words. Milestones: ch11 closed 100% (371-410); staging bank CHOROID_STAGING_EXTRACTS.md sections A-K | v1.1.0 article enrichment 2026-10-27: 3 fields extended (+224 words) from 2 verified articles — Nickla &amp; Wallman 2010 Prog Retin Eye Res 29(2):144-168 (flow 10x brain/thermoregulation/retinal-position adjustment/growth-factor secretion + emmetropization) + Margolis &amp; Spaide 2009 AJO 147(5):811-815 (EDI-OCT subfoveal 287±76µm, −15.6µm/decade); validate 46/46 + pytest 10+14 green (2026-10-27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>CHO-002</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Choroid</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Choroidal Layers (Haller / Sattler / choriocapillaris / Bruch's membrane)</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>14,17</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>ch11: 377-378, 393-398, 409-410; ch14: 460-464; ch17: 640 | Bruch's five layers 0.3/1/-/-/0.14um (397-398); RPE produces type IV collagen/heparan sulphate/laminin into lamina vitrea (464); Bruch stops abruptly at disc + choroidal ring (460); melanosomes 0.3-0.4um always &lt; RPE (378); musculo-elastic system + pericytes 1:6; drusen &gt;40y (398); 4 of 5 Bruch layers by week 9, outermost last (640); ageing sheaths Tripathi &amp; Tripathi 1974 (410)</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>choroid-layers.json</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff ch.11 + ch14 RPE section + ch17 development)</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 46/46, 2026-10-27)</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>v1.0.0; created 2026-10-27. 8/8 fields documented, 1,047 words. layers array = 4 items with full Bruch's five-layer breakdown | v1.1.0 article enrichment 2026-10-27: 2 fields extended (+141 words) — Ramrattan 1994 IOVS 35(6):2857-64 (Bruch +135% 2.0→4.7µm; choroid −57% 193.5→84µm; AMD BLD/GA/disciform density 63/54/43% of normal) + Nivison-Smith 2020 Sci Rep 10:10810 (eccentricity- and age-dependent angioarchitecture); validate 46/46 + pytest 10+14 green (2026-10-27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>CHO-003</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Choroid</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Choriocapillaris (fenestrated net, lobular organization, permeability)</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>7,14,15,17</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>ch11: 377-378, 384-396, 408-410; ch14: 455; ch15: 500,534-535; ch17: 637-638 | lobules arteriocentric Hayreh vs venocentric Fryczkowski (392); lobule sizes 515x450 posterior / 645x550 equator / 955x670 periphery, ratios 1:1 submacular to 1:5 (385); fenestrations 60-80nm (396); leaky junctions hepatic-sinusoid-like; pericytes 1:6 scleral aspect (395); protein leak 5x kidney 10x muscle + osmotic 15mmHg (408); cherry-red spot mechanism (455); no BBB across fenestrated capillaries at disc (500,534); unchanged in glaucoma until long-standing (410); development: only mesoderm touching RPE forms net, fenestrations after week 7 (637-638)</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>choriocapillaris.json</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff ch.11 + ch14 foveola + ch15 disc + ch17)</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 46/46, 2026-10-27)</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>v1.0.0; created 2026-10-27. 7/8 fields documented (layers not_applicable), 892 words | v1.1.0 article enrichment 2026-10-27: 3 fields extended (+214 words) — Fryczkowski 1991 Int Ophthalmol 15(2):109-120 (casts; regional angioarchitecture) + Zouache 2016 Sci Rep 6:35754 (segmented-flow tessellation) + Ramrattan 1994 (density −45%; diameter −34% 9.8→6.5µm) + Nickla 2010 (flow 10x brain); validate 46/46 + pytest 10+14 green (2026-10-27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>CHO-004</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Choroid</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Choroidal Blood Supply (SPCA/LPCA/ACA system, Zinn-Haller, territories)</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>3,15,17</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>ch11: 371-376, 384-393, 406-407; ch3: 88; ch15: 528-534,570; ch17: 638-639 | 10-20 SPCAs (371,88); Zinn-Haller frequency dispute Olver 1990 vs Hayreh 1964, absent in sub-human primates (371-373,529-531); LPCA oblique 4mm canal + 45-degree bend + blue-line landmark (373); recurrent choroidal branches towards equator (531); lateral PCA up to 2/3 of choroid + vertical watershed (393); anterior segment ischaemia after recti disinsertion/bands (376); Amalric triangles + Elschnig spots (393); disc supply 10%/30% prelaminar Lieberman 1976 (534); Ruskell 1984 interfacial precapillaries - glaucoma disc haemorrhages (531); development final anastomosis month 8 (639)</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>choroid-blood-supply.json</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff ch.11 + ch3 origin + ch15 optic nerve head supply + ch17)</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 46/46, 2026-10-27)</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>v1.0.0; created 2026-10-27. 8/8 fields documented, 1,028 words. layers array = 6-tier arterial cascade | v1.1.0 article enrichment 2026-10-27: 1 field extended (+110 words) — Alm &amp; Bill 1973 Exp Eye Res 15(1):15-29 registered as the standard microsphere/no-autoregulation anchor + Reiner 2018 Prog Retin Eye Res 64:96-130 + Nickla 2010; validate 46/46 + pytest 10+14 green (2026-10-27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>CHO-005</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Choroid</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Vortex Veins (venae vorticosae — ampullae, sectors, drainage)</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>3,7,17</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>ch11: 224, 405-407; ch7: 274; ch3: 101 | Rutnin 1967: visible ~90%, ampulliform ~50%, 8 (4-15) enter / 6 (5-8, mean 5.82) exit, intrascleral course 4.53mm (1.25-8.5) (224); Table 7.2 limbus distances 22/18, 20/16, 19/15, 18/14.5 (274); exits ~6mm behind equator, superolateral 8mm, inferolateral 5.5mm (405); whorl visible in blond/myopic/albinoid fundi (406); sectorial drainage iris-to-choroid + Maltese cross watershed crossing submacular choroid (Hayreh &amp; Baines 1973 BJO 57,217) (406-407); SOV first/third part + IOV positional anastomosis (406,101); valveless; development month 2 (638)</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>vortex-veins.json</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff ch.11 veins section + ch7 Table 7.2 + ch3 orbital veins + ch17)</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 46/46, 2026-10-27)</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>v1.0.0; created 2026-10-27. 7/8 fields documented (layers not_applicable), 780 words | v1.1.0 article enrichment 2026-10-27: 2 fields extended (+163 words) — Verma 2021 Clin Ophthalmol 15:3321 (4-8 vortices; 4:35%/5:30%; UWFA mean 8; SOV→cavernous sinus / IOV→pterygoid plexus; pachychoroid) + Lim 1995 Ophthalmology 102(6):942-946 (scleral exit coordinates) + Hayreh &amp; Baines 1973 BJO 57(4):217 full text registered; validate 46/46 + pytest 10+14 green (2026-10-27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>CHO-006</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Choroid</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Suprachoroidal Space (lamina suprachoroidea, lamina fusca, outflow)</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>7,8,15</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>ch11: 373, 376-377, 502; ch7: 274-276; ch8: 302 | thickness 10-34um (377); posterior lamellae adherent -&gt; detachments anteriorly rarely cross equator + sonar sees effusion without ballooning (377); musculo-elastic system + posterior elastic tendon of ciliary muscle (Rohen/Tamm/Lutjen-Drecoll 1995) (377); myofibroblasts = muscle spindles of Salzmann, compliant pillow hypothesis (377); lamina fusca melanocytes -&gt; deep scleral pigmentation (276); uveoscleral/uveovortex outflow (302); meridional lamellae + denser pigment near optic nerve (502)</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>suprachoroidal-space.json</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff ch.11 suprachoroidea + ch7 sclera + ch8 angle + ch15 disc relations)</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 46/46, 2026-10-27)</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>v1.0.0; created 2026-10-27. 8/8 fields documented, 731 words. layers array = 5 structural components | v1.1.0 article enrichment 2026-10-27: 2 fields extended (+109 words) — Chiang, Jung &amp; Prausnitz 2018 Adv Drug Deliv Rev 126:58-66 (SCS potential space; high bioavailability to choroid/RPE/retina; microneedle access; phase III trials); validate 46/46 + pytest 10+14 green (2026-10-27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>CHO-007</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Choroid</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Choroidal Innervation (dual autonomic + intrinsic nitrergic plexus)</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Wolff</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>ch11: 383-384, 408-410; ch16: 606-619 | dual supply: sympathetic vasoconstrictor tone (Bill/Linder 1977b) + parasympathetic by TWO routes - III via ciliary ganglion and facial via pterygopalatine (383); intrinsic nitrergic/VIPergic plexus ~2000 cells, foveate species only, submacular concentration = light protection (Flugel 1994) (383-384); no innervation on choriocapillaris (Ruskell 1971b); rami oculares: ~27 rami, 12x8um, ~24 bundles x 56 axons, no sympathetic fibres (606); coexpressed muscarinic+VIPergic+nitrergic; pterygopalatine ganglionectomy -&gt; IOP fall, greater petrosal stimulation -&gt; IOP rise Gloster 1961 (607); CHOROIDAL VESSELS summary section (619); glaucoma ganglion-cell loss parallel to thinning (410)</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>choroid-innervation.json</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Done (manual, Wolff ch.11 innervation + circulation + ch16 autonomic chapter)</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>Yes (validate.py, 46/46, 2026-10-27)</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>Z.ai assistant</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>v1.0.0; created 2026-10-27. 5/8 fields documented (layers/blood_supply/venous_drainage not_applicable), 839 words — the innervation field is the richest in the KB (autonomic triple coexpression documented) | v1.1.0 article enrichment 2026-10-27: 2 fields extended (+166 words) — Reiner 2018 Prog Retin Eye Res 64:96-130 (parasympathetic vasodilator / sympathetic vasoconstrictor / trigeminal sensory dual role; impairments in aging, glaucoma, AMD, HTN, diabetes); validate 46/46 + pytest 10+14 green (2026-10-27)</t>
         </is>
       </c>
     </row>

</xml_diff>